<commit_message>
update template simple audit
</commit_message>
<xml_diff>
--- a/src/files/en/general/template-grille-audit-simplifie.xlsx
+++ b/src/files/en/general/template-grille-audit-simplifie.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\IFI774\ProjectsACC\accessibilite.public.lu\src\files\en\general\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VUJ787\Documents\Audit simplifiés\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2454FF93-992A-445D-9334-E633200B402A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7C40FCFC-3386-46E5-89B5-507DB3176649}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" tabRatio="861" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="861" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sample" sheetId="2" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="624" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="783" uniqueCount="187">
   <si>
     <t>Site :</t>
   </si>
@@ -602,6 +602,12 @@
   </si>
   <si>
     <t>On each web page, is every moving or blinking content controllable by the user?</t>
+  </si>
+  <si>
+    <t>In each form, is the error managementl used appropriately (excluding special cases)?</t>
+  </si>
+  <si>
+    <t>Can content grouping regions present in several web pages (header, main navigation, main content, footer and search engine) be reached or avoided?</t>
   </si>
 </sst>
 </file>
@@ -1511,15 +1517,6 @@
     <xf numFmtId="0" fontId="11" fillId="9" borderId="0" xfId="12" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="23" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="24" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="25" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="8" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
@@ -1532,25 +1529,34 @@
     <xf numFmtId="0" fontId="11" fillId="9" borderId="2" xfId="12" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="23" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="24" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="25" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="3" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="3" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="18" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="21" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="20" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="22" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="18" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="21" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="22" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="20" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="9" borderId="2" xfId="12" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1670,6 +1676,34 @@
       <font>
         <b/>
         <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <name val="Arial"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFFCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <sz val="12"/>
         <color rgb="FFFFFFFF"/>
         <name val="Arial"/>
       </font>
@@ -1719,34 +1753,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FF07838B"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <name val="Arial"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFFFCC"/>
         </patternFill>
       </fill>
     </dxf>
@@ -7564,12 +7570,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="94" t="str">
+      <c r="A1" s="98" t="str">
         <f>Sample!A1</f>
         <v>SIMPLIFIED AUDIT – ASSESSMENT GRID</v>
       </c>
-      <c r="B1" s="95"/>
-      <c r="C1" s="96"/>
+      <c r="B1" s="99"/>
+      <c r="C1" s="100"/>
     </row>
     <row r="2" spans="1:4" ht="70.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="29" t="s">
@@ -7583,7 +7589,7 @@
       </c>
     </row>
     <row r="3" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A3" s="97" t="s">
+      <c r="A3" s="94" t="s">
         <v>5</v>
       </c>
       <c r="B3" s="57" t="s">
@@ -7595,7 +7601,7 @@
       <c r="D3" s="6"/>
     </row>
     <row r="4" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A4" s="97"/>
+      <c r="A4" s="94"/>
       <c r="B4" s="57" t="s">
         <v>7</v>
       </c>
@@ -7605,7 +7611,7 @@
       <c r="D4" s="6"/>
     </row>
     <row r="5" spans="1:4" ht="30" x14ac:dyDescent="0.2">
-      <c r="A5" s="97"/>
+      <c r="A5" s="94"/>
       <c r="B5" s="57" t="s">
         <v>8</v>
       </c>
@@ -7615,7 +7621,7 @@
       <c r="D5" s="6"/>
     </row>
     <row r="6" spans="1:4" ht="30" x14ac:dyDescent="0.2">
-      <c r="A6" s="97"/>
+      <c r="A6" s="94"/>
       <c r="B6" s="57" t="s">
         <v>9</v>
       </c>
@@ -7625,7 +7631,7 @@
       <c r="D6" s="6"/>
     </row>
     <row r="7" spans="1:4" ht="30" x14ac:dyDescent="0.2">
-      <c r="A7" s="97"/>
+      <c r="A7" s="94"/>
       <c r="B7" s="57" t="s">
         <v>10</v>
       </c>
@@ -7635,7 +7641,7 @@
       <c r="D7" s="6"/>
     </row>
     <row r="8" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A8" s="97"/>
+      <c r="A8" s="94"/>
       <c r="B8" s="57" t="s">
         <v>11</v>
       </c>
@@ -7645,7 +7651,7 @@
       <c r="D8" s="6"/>
     </row>
     <row r="9" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A9" s="97"/>
+      <c r="A9" s="94"/>
       <c r="B9" s="57" t="s">
         <v>12</v>
       </c>
@@ -7667,7 +7673,7 @@
       <c r="D10" s="6"/>
     </row>
     <row r="11" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A11" s="97" t="s">
+      <c r="A11" s="94" t="s">
         <v>118</v>
       </c>
       <c r="B11" s="57" t="s">
@@ -7679,7 +7685,7 @@
       <c r="D11" s="6"/>
     </row>
     <row r="12" spans="1:4" ht="30" x14ac:dyDescent="0.2">
-      <c r="A12" s="97"/>
+      <c r="A12" s="94"/>
       <c r="B12" s="57" t="s">
         <v>16</v>
       </c>
@@ -7689,7 +7695,7 @@
       <c r="D12" s="6"/>
     </row>
     <row r="13" spans="1:4" ht="30" x14ac:dyDescent="0.2">
-      <c r="A13" s="97" t="s">
+      <c r="A13" s="94" t="s">
         <v>119</v>
       </c>
       <c r="B13" s="57" t="s">
@@ -7701,7 +7707,7 @@
       <c r="D13" s="6"/>
     </row>
     <row r="14" spans="1:4" ht="30" x14ac:dyDescent="0.2">
-      <c r="A14" s="97"/>
+      <c r="A14" s="94"/>
       <c r="B14" s="57" t="s">
         <v>19</v>
       </c>
@@ -7711,7 +7717,7 @@
       <c r="D14" s="6"/>
     </row>
     <row r="15" spans="1:4" ht="30" x14ac:dyDescent="0.2">
-      <c r="A15" s="97"/>
+      <c r="A15" s="94"/>
       <c r="B15" s="57" t="s">
         <v>20</v>
       </c>
@@ -7721,7 +7727,7 @@
       <c r="D15" s="6"/>
     </row>
     <row r="16" spans="1:4" ht="30" x14ac:dyDescent="0.2">
-      <c r="A16" s="97"/>
+      <c r="A16" s="94"/>
       <c r="B16" s="57" t="s">
         <v>21</v>
       </c>
@@ -7731,7 +7737,7 @@
       <c r="D16" s="6"/>
     </row>
     <row r="17" spans="1:64" ht="15" x14ac:dyDescent="0.2">
-      <c r="A17" s="97"/>
+      <c r="A17" s="94"/>
       <c r="B17" s="57" t="s">
         <v>22</v>
       </c>
@@ -7741,7 +7747,7 @@
       <c r="D17" s="6"/>
     </row>
     <row r="18" spans="1:64" ht="15" x14ac:dyDescent="0.2">
-      <c r="A18" s="97"/>
+      <c r="A18" s="94"/>
       <c r="B18" s="57" t="s">
         <v>23</v>
       </c>
@@ -7751,7 +7757,7 @@
       <c r="D18" s="6"/>
     </row>
     <row r="19" spans="1:64" ht="15" x14ac:dyDescent="0.2">
-      <c r="A19" s="97"/>
+      <c r="A19" s="94"/>
       <c r="B19" s="57" t="s">
         <v>24</v>
       </c>
@@ -7761,7 +7767,7 @@
       <c r="D19" s="6"/>
     </row>
     <row r="20" spans="1:64" ht="15" x14ac:dyDescent="0.2">
-      <c r="A20" s="97"/>
+      <c r="A20" s="94"/>
       <c r="B20" s="57" t="s">
         <v>25</v>
       </c>
@@ -7771,7 +7777,7 @@
       <c r="D20" s="6"/>
     </row>
     <row r="21" spans="1:64" ht="15" x14ac:dyDescent="0.2">
-      <c r="A21" s="97" t="s">
+      <c r="A21" s="94" t="s">
         <v>120</v>
       </c>
       <c r="B21" s="57" t="s">
@@ -7783,7 +7789,7 @@
       <c r="D21" s="6"/>
     </row>
     <row r="22" spans="1:64" ht="30" x14ac:dyDescent="0.2">
-      <c r="A22" s="97"/>
+      <c r="A22" s="94"/>
       <c r="B22" s="57" t="s">
         <v>28</v>
       </c>
@@ -7793,7 +7799,7 @@
       <c r="D22" s="6"/>
     </row>
     <row r="23" spans="1:64" ht="15" x14ac:dyDescent="0.2">
-      <c r="A23" s="97" t="s">
+      <c r="A23" s="94" t="s">
         <v>121</v>
       </c>
       <c r="B23" s="57" t="s">
@@ -7805,7 +7811,7 @@
       <c r="D23" s="6"/>
     </row>
     <row r="24" spans="1:64" ht="15" x14ac:dyDescent="0.2">
-      <c r="A24" s="97"/>
+      <c r="A24" s="94"/>
       <c r="B24" s="57" t="s">
         <v>31</v>
       </c>
@@ -7896,7 +7902,7 @@
       <c r="BL26" s="5"/>
     </row>
     <row r="27" spans="1:64" s="3" customFormat="1" ht="15" x14ac:dyDescent="0.2">
-      <c r="A27" s="98" t="s">
+      <c r="A27" s="95" t="s">
         <v>122</v>
       </c>
       <c r="B27" s="31" t="s">
@@ -7967,7 +7973,7 @@
       <c r="BL27" s="5"/>
     </row>
     <row r="28" spans="1:64" s="3" customFormat="1" ht="15" x14ac:dyDescent="0.2">
-      <c r="A28" s="99"/>
+      <c r="A28" s="96"/>
       <c r="B28" s="31" t="s">
         <v>86</v>
       </c>
@@ -8036,7 +8042,7 @@
       <c r="BL28" s="5"/>
     </row>
     <row r="29" spans="1:64" ht="15" x14ac:dyDescent="0.2">
-      <c r="A29" s="99"/>
+      <c r="A29" s="96"/>
       <c r="B29" s="57" t="s">
         <v>35</v>
       </c>
@@ -8046,7 +8052,7 @@
       <c r="D29" s="6"/>
     </row>
     <row r="30" spans="1:64" ht="15" x14ac:dyDescent="0.2">
-      <c r="A30" s="99"/>
+      <c r="A30" s="96"/>
       <c r="B30" s="57" t="s">
         <v>36</v>
       </c>
@@ -8056,7 +8062,7 @@
       <c r="D30" s="6"/>
     </row>
     <row r="31" spans="1:64" ht="15" x14ac:dyDescent="0.2">
-      <c r="A31" s="99"/>
+      <c r="A31" s="96"/>
       <c r="B31" s="57" t="s">
         <v>37</v>
       </c>
@@ -8066,7 +8072,7 @@
       <c r="D31" s="6"/>
     </row>
     <row r="32" spans="1:64" ht="15" x14ac:dyDescent="0.2">
-      <c r="A32" s="99"/>
+      <c r="A32" s="96"/>
       <c r="B32" s="57" t="s">
         <v>38</v>
       </c>
@@ -8076,7 +8082,7 @@
       <c r="D32" s="6"/>
     </row>
     <row r="33" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A33" s="100"/>
+      <c r="A33" s="97"/>
       <c r="B33" s="57" t="s">
         <v>39</v>
       </c>
@@ -8086,7 +8092,7 @@
       <c r="D33" s="6"/>
     </row>
     <row r="34" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A34" s="97" t="s">
+      <c r="A34" s="94" t="s">
         <v>40</v>
       </c>
       <c r="B34" s="57" t="s">
@@ -8098,7 +8104,7 @@
       <c r="D34" s="6"/>
     </row>
     <row r="35" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A35" s="97"/>
+      <c r="A35" s="94"/>
       <c r="B35" s="57" t="s">
         <v>42</v>
       </c>
@@ -8108,7 +8114,7 @@
       <c r="D35" s="6"/>
     </row>
     <row r="36" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A36" s="97" t="s">
+      <c r="A36" s="94" t="s">
         <v>123</v>
       </c>
       <c r="B36" s="57" t="s">
@@ -8120,7 +8126,7 @@
       <c r="D36" s="6"/>
     </row>
     <row r="37" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A37" s="97"/>
+      <c r="A37" s="94"/>
       <c r="B37" s="57" t="s">
         <v>45</v>
       </c>
@@ -8130,7 +8136,7 @@
       <c r="D37" s="6"/>
     </row>
     <row r="38" spans="1:4" ht="30" x14ac:dyDescent="0.2">
-      <c r="A38" s="97"/>
+      <c r="A38" s="94"/>
       <c r="B38" s="57" t="s">
         <v>46</v>
       </c>
@@ -8140,7 +8146,7 @@
       <c r="D38" s="6"/>
     </row>
     <row r="39" spans="1:4" ht="30" x14ac:dyDescent="0.2">
-      <c r="A39" s="97"/>
+      <c r="A39" s="94"/>
       <c r="B39" s="57" t="s">
         <v>47</v>
       </c>
@@ -8150,7 +8156,7 @@
       <c r="D39" s="6"/>
     </row>
     <row r="40" spans="1:4" ht="30" x14ac:dyDescent="0.2">
-      <c r="A40" s="97"/>
+      <c r="A40" s="94"/>
       <c r="B40" s="57" t="s">
         <v>48</v>
       </c>
@@ -8160,7 +8166,7 @@
       <c r="D40" s="6"/>
     </row>
     <row r="41" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A41" s="97" t="s">
+      <c r="A41" s="94" t="s">
         <v>124</v>
       </c>
       <c r="B41" s="57" t="s">
@@ -8172,7 +8178,7 @@
       <c r="D41" s="6"/>
     </row>
     <row r="42" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A42" s="97"/>
+      <c r="A42" s="94"/>
       <c r="B42" s="57" t="s">
         <v>51</v>
       </c>
@@ -8182,7 +8188,7 @@
       <c r="D42" s="6"/>
     </row>
     <row r="43" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A43" s="97"/>
+      <c r="A43" s="94"/>
       <c r="B43" s="57" t="s">
         <v>52</v>
       </c>
@@ -8192,7 +8198,7 @@
       <c r="D43" s="6"/>
     </row>
     <row r="44" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A44" s="97"/>
+      <c r="A44" s="94"/>
       <c r="B44" s="57" t="s">
         <v>53</v>
       </c>
@@ -8202,7 +8208,7 @@
       <c r="D44" s="6"/>
     </row>
     <row r="45" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A45" s="97"/>
+      <c r="A45" s="94"/>
       <c r="B45" s="57" t="s">
         <v>54</v>
       </c>
@@ -8212,7 +8218,7 @@
       <c r="D45" s="6"/>
     </row>
     <row r="46" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A46" s="97"/>
+      <c r="A46" s="94"/>
       <c r="B46" s="57" t="s">
         <v>55</v>
       </c>
@@ -8222,7 +8228,7 @@
       <c r="D46" s="6"/>
     </row>
     <row r="47" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A47" s="97"/>
+      <c r="A47" s="94"/>
       <c r="B47" s="57" t="s">
         <v>56</v>
       </c>
@@ -8232,7 +8238,7 @@
       <c r="D47" s="6"/>
     </row>
     <row r="48" spans="1:4" ht="30" x14ac:dyDescent="0.2">
-      <c r="A48" s="97" t="s">
+      <c r="A48" s="94" t="s">
         <v>57</v>
       </c>
       <c r="B48" s="57" t="s">
@@ -8244,7 +8250,7 @@
       <c r="D48" s="6"/>
     </row>
     <row r="49" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A49" s="97"/>
+      <c r="A49" s="94"/>
       <c r="B49" s="57" t="s">
         <v>59</v>
       </c>
@@ -8254,7 +8260,7 @@
       <c r="D49" s="6"/>
     </row>
     <row r="50" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A50" s="97"/>
+      <c r="A50" s="94"/>
       <c r="B50" s="57" t="s">
         <v>60</v>
       </c>
@@ -8264,7 +8270,7 @@
       <c r="D50" s="6"/>
     </row>
     <row r="51" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A51" s="97"/>
+      <c r="A51" s="94"/>
       <c r="B51" s="57" t="s">
         <v>61</v>
       </c>
@@ -8274,7 +8280,7 @@
       <c r="D51" s="6"/>
     </row>
     <row r="52" spans="1:4" ht="30" x14ac:dyDescent="0.2">
-      <c r="A52" s="97"/>
+      <c r="A52" s="94"/>
       <c r="B52" s="57" t="s">
         <v>62</v>
       </c>
@@ -8284,7 +8290,7 @@
       <c r="D52" s="6"/>
     </row>
     <row r="53" spans="1:4" ht="30" x14ac:dyDescent="0.2">
-      <c r="A53" s="97" t="s">
+      <c r="A53" s="94" t="s">
         <v>63</v>
       </c>
       <c r="B53" s="57" t="s">
@@ -8296,7 +8302,7 @@
       <c r="D53" s="6"/>
     </row>
     <row r="54" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A54" s="97"/>
+      <c r="A54" s="94"/>
       <c r="B54" s="57" t="s">
         <v>65</v>
       </c>
@@ -8306,7 +8312,7 @@
       <c r="D54" s="6"/>
     </row>
     <row r="55" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A55" s="97"/>
+      <c r="A55" s="94"/>
       <c r="B55" s="57" t="s">
         <v>66</v>
       </c>
@@ -8317,6 +8323,11 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A3:A9"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A13:A20"/>
+    <mergeCell ref="A36:A40"/>
     <mergeCell ref="A41:A47"/>
     <mergeCell ref="A48:A52"/>
     <mergeCell ref="A53:A55"/>
@@ -8324,11 +8335,6 @@
     <mergeCell ref="A23:A24"/>
     <mergeCell ref="A34:A35"/>
     <mergeCell ref="A27:A33"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A3:A9"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A13:A20"/>
-    <mergeCell ref="A36:A40"/>
   </mergeCells>
   <pageMargins left="0.39374999999999999" right="0.39374999999999999" top="0.53263888888888899" bottom="0.39374999999999999" header="0.39374999999999999" footer="0.39374999999999999"/>
   <pageSetup scale="74" pageOrder="overThenDown" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -9214,7 +9220,7 @@
       <c r="BL3" s="2"/>
     </row>
     <row r="4" spans="1:1023" ht="30" x14ac:dyDescent="0.2">
-      <c r="A4" s="105" t="str">
+      <c r="A4" s="106" t="str">
         <f>Criteria!$A$3</f>
         <v>IMAGES</v>
       </c>
@@ -9222,9 +9228,8 @@
         <f>Criteria!B3</f>
         <v>1.1</v>
       </c>
-      <c r="C4" s="32" t="str">
-        <f>Criteria!C3</f>
-        <v>Does each image conveying information have a text alternative?</v>
+      <c r="C4" s="32" t="s">
+        <v>125</v>
       </c>
       <c r="D4" s="32" t="s">
         <v>73</v>
@@ -9293,14 +9298,13 @@
       <c r="BL4" s="2"/>
     </row>
     <row r="5" spans="1:1023" ht="30" x14ac:dyDescent="0.2">
-      <c r="A5" s="105"/>
+      <c r="A5" s="106"/>
       <c r="B5" s="46" t="str">
         <f>Criteria!B4</f>
         <v>1.2</v>
       </c>
-      <c r="C5" s="32" t="str">
-        <f>Criteria!C4</f>
-        <v>Is every decorative image correctly ignored by assistive technologies?</v>
+      <c r="C5" s="32" t="s">
+        <v>126</v>
       </c>
       <c r="D5" s="32" t="s">
         <v>73</v>
@@ -9375,14 +9379,13 @@
       <c r="AMI5" s="14"/>
     </row>
     <row r="6" spans="1:1023" ht="45" x14ac:dyDescent="0.2">
-      <c r="A6" s="105"/>
+      <c r="A6" s="106"/>
       <c r="B6" s="46" t="str">
         <f>Criteria!B5</f>
         <v>1.3</v>
       </c>
-      <c r="C6" s="32" t="str">
-        <f>Criteria!C5</f>
-        <v>For each image conveying information with a text alternative, is this alternative relevant (excluding special cases)?</v>
+      <c r="C6" s="32" t="s">
+        <v>127</v>
       </c>
       <c r="D6" s="32" t="s">
         <v>73</v>
@@ -9451,14 +9454,13 @@
       <c r="BL6" s="2"/>
     </row>
     <row r="7" spans="1:1023" ht="45" x14ac:dyDescent="0.2">
-      <c r="A7" s="105"/>
+      <c r="A7" s="106"/>
       <c r="B7" s="46" t="str">
         <f>Criteria!B6</f>
         <v>1.4</v>
       </c>
-      <c r="C7" s="32" t="str">
-        <f>Criteria!C6</f>
-        <v>For each image used as a CAPTCHA or test image, with a text alternative, does this alternative make it possible to identify the nature and function of the image?</v>
+      <c r="C7" s="32" t="s">
+        <v>128</v>
       </c>
       <c r="D7" s="32" t="s">
         <v>73</v>
@@ -9470,14 +9472,13 @@
       <c r="G7" s="32"/>
     </row>
     <row r="8" spans="1:1023" ht="45" x14ac:dyDescent="0.2">
-      <c r="A8" s="105"/>
+      <c r="A8" s="106"/>
       <c r="B8" s="46" t="str">
         <f>Criteria!B7</f>
         <v>1.5</v>
       </c>
-      <c r="C8" s="32" t="str">
-        <f>Criteria!C7</f>
-        <v>For each image used as a CAPTCHA, is there an alternative access solution to the content or to the CAPTCHA function?</v>
+      <c r="C8" s="32" t="s">
+        <v>129</v>
       </c>
       <c r="D8" s="32" t="s">
         <v>73</v>
@@ -9489,14 +9490,13 @@
       <c r="G8" s="32"/>
     </row>
     <row r="9" spans="1:1023" ht="30" x14ac:dyDescent="0.2">
-      <c r="A9" s="105"/>
+      <c r="A9" s="106"/>
       <c r="B9" s="46" t="str">
         <f>Criteria!B8</f>
         <v>1.6</v>
       </c>
-      <c r="C9" s="32" t="str">
-        <f>Criteria!C8</f>
-        <v>Does each image conveying information have, if necessary, a detailed description?</v>
+      <c r="C9" s="32" t="s">
+        <v>130</v>
       </c>
       <c r="D9" s="32" t="s">
         <v>73</v>
@@ -9508,14 +9508,13 @@
       <c r="G9" s="32"/>
     </row>
     <row r="10" spans="1:1023" ht="30" x14ac:dyDescent="0.2">
-      <c r="A10" s="97"/>
+      <c r="A10" s="94"/>
       <c r="B10" s="74" t="str">
         <f>Criteria!B9</f>
         <v>1.7</v>
       </c>
-      <c r="C10" s="75" t="str">
-        <f>Criteria!C9</f>
-        <v>For each image conveying information with a detailed description, is this description relevant?</v>
+      <c r="C10" s="75" t="s">
+        <v>131</v>
       </c>
       <c r="D10" s="32" t="s">
         <v>73</v>
@@ -9535,9 +9534,8 @@
         <f>Criteria!B10</f>
         <v>2.1</v>
       </c>
-      <c r="C11" s="80" t="str">
-        <f>Criteria!C10</f>
-        <v>Does each frame have a frame title?</v>
+      <c r="C11" s="80" t="s">
+        <v>132</v>
       </c>
       <c r="D11" s="32" t="s">
         <v>73</v>
@@ -9549,7 +9547,7 @@
       <c r="G11" s="80"/>
     </row>
     <row r="12" spans="1:1023" ht="30" x14ac:dyDescent="0.2">
-      <c r="A12" s="99" t="str">
+      <c r="A12" s="96" t="str">
         <f>Criteria!$A$11</f>
         <v>COLOURS</v>
       </c>
@@ -9557,9 +9555,8 @@
         <f>Criteria!B11</f>
         <v>3.1</v>
       </c>
-      <c r="C12" s="77" t="str">
-        <f>Criteria!C11</f>
-        <v>On each web page, the information must not be provided by colour alone. Is this rule respected?</v>
+      <c r="C12" s="77" t="s">
+        <v>169</v>
       </c>
       <c r="D12" s="32" t="s">
         <v>73</v>
@@ -9571,14 +9568,13 @@
       <c r="G12" s="77"/>
     </row>
     <row r="13" spans="1:1023" ht="45" x14ac:dyDescent="0.2">
-      <c r="A13" s="97"/>
+      <c r="A13" s="94"/>
       <c r="B13" s="74" t="str">
         <f>Criteria!B12</f>
         <v>3.2</v>
       </c>
-      <c r="C13" s="75" t="str">
-        <f>Criteria!C12</f>
-        <v>On each web page, is the contrast between the colour of the text and the colour of its background sufficiently high (excluding special cases)?</v>
+      <c r="C13" s="75" t="s">
+        <v>133</v>
       </c>
       <c r="D13" s="32" t="s">
         <v>73</v>
@@ -9590,7 +9586,7 @@
       <c r="G13" s="75"/>
     </row>
     <row r="14" spans="1:1023" ht="45" x14ac:dyDescent="0.2">
-      <c r="A14" s="103" t="str">
+      <c r="A14" s="105" t="str">
         <f>Criteria!$A$13</f>
         <v>MULTIMEDIA</v>
       </c>
@@ -9598,9 +9594,8 @@
         <f>Criteria!B13</f>
         <v>4.1</v>
       </c>
-      <c r="C14" s="82" t="str">
-        <f>Criteria!C13</f>
-        <v>Does each pre-recorded time-based media have, if necessary, a transcript or an audio description (excluding special cases)?</v>
+      <c r="C14" s="82" t="s">
+        <v>134</v>
       </c>
       <c r="D14" s="32" t="s">
         <v>73</v>
@@ -9612,14 +9607,13 @@
       <c r="G14" s="82"/>
     </row>
     <row r="15" spans="1:1023" ht="45" x14ac:dyDescent="0.2">
-      <c r="A15" s="105"/>
+      <c r="A15" s="106"/>
       <c r="B15" s="46" t="str">
         <f>Criteria!B14</f>
         <v>4.2</v>
       </c>
-      <c r="C15" s="32" t="str">
-        <f>Criteria!C14</f>
-        <v>For each pre-recorded time-based media with a synchronised transcript or audio description, are these relevant (excluding special cases)?</v>
+      <c r="C15" s="32" t="s">
+        <v>135</v>
       </c>
       <c r="D15" s="32" t="s">
         <v>73</v>
@@ -9631,14 +9625,13 @@
       <c r="G15" s="32"/>
     </row>
     <row r="16" spans="1:1023" ht="45" x14ac:dyDescent="0.2">
-      <c r="A16" s="105"/>
+      <c r="A16" s="106"/>
       <c r="B16" s="46" t="str">
         <f>Criteria!B15</f>
         <v>4.3</v>
       </c>
-      <c r="C16" s="32" t="str">
-        <f>Criteria!C15</f>
-        <v>Does each pre-recorded synchronised time-based media have, if necessary, synchronised captions (excluding special cases)?</v>
+      <c r="C16" s="32" t="s">
+        <v>170</v>
       </c>
       <c r="D16" s="32" t="s">
         <v>73</v>
@@ -9650,14 +9643,13 @@
       <c r="G16" s="32"/>
     </row>
     <row r="17" spans="1:64" ht="45" x14ac:dyDescent="0.2">
-      <c r="A17" s="105"/>
+      <c r="A17" s="106"/>
       <c r="B17" s="46" t="str">
         <f>Criteria!B16</f>
         <v>4.4</v>
       </c>
-      <c r="C17" s="32" t="str">
-        <f>Criteria!C16</f>
-        <v>For each pre-recorded synchronised time-based media with synchronised subtitles, are these captions relevant?</v>
+      <c r="C17" s="32" t="s">
+        <v>171</v>
       </c>
       <c r="D17" s="32" t="s">
         <v>73</v>
@@ -9669,14 +9661,13 @@
       <c r="G17" s="32"/>
     </row>
     <row r="18" spans="1:64" ht="30" x14ac:dyDescent="0.2">
-      <c r="A18" s="105"/>
+      <c r="A18" s="106"/>
       <c r="B18" s="46" t="str">
         <f>Criteria!B17</f>
         <v>4.8</v>
       </c>
-      <c r="C18" s="32" t="str">
-        <f>Criteria!C17</f>
-        <v>Does each non-time-based media have, if necessary, an alternative (excluding special cases)?</v>
+      <c r="C18" s="32" t="s">
+        <v>136</v>
       </c>
       <c r="D18" s="32" t="s">
         <v>73</v>
@@ -9688,14 +9679,13 @@
       <c r="G18" s="32"/>
     </row>
     <row r="19" spans="1:64" ht="30" x14ac:dyDescent="0.2">
-      <c r="A19" s="105"/>
+      <c r="A19" s="106"/>
       <c r="B19" s="46" t="str">
         <f>Criteria!B18</f>
         <v>4.9</v>
       </c>
-      <c r="C19" s="32" t="str">
-        <f>Criteria!C18</f>
-        <v>For each non-time-based media having an alternative, is this alternative relevant?</v>
+      <c r="C19" s="32" t="s">
+        <v>137</v>
       </c>
       <c r="D19" s="32" t="s">
         <v>73</v>
@@ -9707,14 +9697,13 @@
       <c r="G19" s="32"/>
     </row>
     <row r="20" spans="1:64" ht="30" x14ac:dyDescent="0.2">
-      <c r="A20" s="105"/>
+      <c r="A20" s="106"/>
       <c r="B20" s="46" t="str">
         <f>Criteria!B19</f>
         <v>4.10</v>
       </c>
-      <c r="C20" s="32" t="str">
-        <f>Criteria!C19</f>
-        <v>Is each automatically triggered sound controllable by the user?</v>
+      <c r="C20" s="32" t="s">
+        <v>138</v>
       </c>
       <c r="D20" s="32" t="s">
         <v>73</v>
@@ -9726,14 +9715,13 @@
       <c r="G20" s="32"/>
     </row>
     <row r="21" spans="1:64" ht="30" x14ac:dyDescent="0.2">
-      <c r="A21" s="104"/>
+      <c r="A21" s="107"/>
       <c r="B21" s="84" t="str">
         <f>Criteria!B20</f>
         <v>4.11</v>
       </c>
-      <c r="C21" s="85" t="str">
-        <f>Criteria!C20</f>
-        <v>Is the viewing of each time-based media, if required, controllable by keyboard and any pointing device?</v>
+      <c r="C21" s="85" t="s">
+        <v>139</v>
       </c>
       <c r="D21" s="32" t="s">
         <v>73</v>
@@ -9745,16 +9733,15 @@
       <c r="G21" s="85"/>
     </row>
     <row r="22" spans="1:64" ht="30" x14ac:dyDescent="0.2">
-      <c r="A22" s="103" t="s">
+      <c r="A22" s="105" t="s">
         <v>26</v>
       </c>
       <c r="B22" s="81" t="str">
         <f>Criteria!B21</f>
         <v>5.6</v>
       </c>
-      <c r="C22" s="82" t="str">
-        <f>Criteria!C21</f>
-        <v>For each data table, are each column header and each row header correctly declared?</v>
+      <c r="C22" s="82" t="s">
+        <v>140</v>
       </c>
       <c r="D22" s="32" t="s">
         <v>73</v>
@@ -9766,14 +9753,13 @@
       <c r="G22" s="82"/>
     </row>
     <row r="23" spans="1:64" ht="45" x14ac:dyDescent="0.2">
-      <c r="A23" s="104"/>
+      <c r="A23" s="107"/>
       <c r="B23" s="84" t="str">
         <f>Criteria!B22</f>
         <v>5.7</v>
       </c>
-      <c r="C23" s="85" t="str">
-        <f>Criteria!C22</f>
-        <v>For each data table, is the appropriate technique used to associate each cell with its headers (excluding special cases)?</v>
+      <c r="C23" s="85" t="s">
+        <v>141</v>
       </c>
       <c r="D23" s="32" t="s">
         <v>73</v>
@@ -9785,7 +9771,7 @@
       <c r="G23" s="85"/>
     </row>
     <row r="24" spans="1:64" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A24" s="103" t="str">
+      <c r="A24" s="105" t="str">
         <f>Criteria!$A$23</f>
         <v>LINKS</v>
       </c>
@@ -9793,9 +9779,8 @@
         <f>Criteria!B23</f>
         <v>6.1</v>
       </c>
-      <c r="C24" s="82" t="str">
-        <f>Criteria!C23</f>
-        <v>Is every link explicit (except in special cases)?</v>
+      <c r="C24" s="82" t="s">
+        <v>142</v>
       </c>
       <c r="D24" s="32" t="s">
         <v>73</v>
@@ -9807,14 +9792,13 @@
       <c r="G24" s="82"/>
     </row>
     <row r="25" spans="1:64" ht="30" x14ac:dyDescent="0.2">
-      <c r="A25" s="104"/>
+      <c r="A25" s="107"/>
       <c r="B25" s="84" t="str">
         <f>Criteria!B24</f>
         <v>6.2</v>
       </c>
-      <c r="C25" s="85" t="str">
-        <f>Criteria!C24</f>
-        <v>On each web page, does each link have an accessible name?</v>
+      <c r="C25" s="85" t="s">
+        <v>172</v>
       </c>
       <c r="D25" s="32" t="s">
         <v>73</v>
@@ -9833,9 +9817,8 @@
         <f>Criteria!B25</f>
         <v>7.3</v>
       </c>
-      <c r="C26" s="80" t="str">
-        <f>Criteria!C25</f>
-        <v>Is each script accessible and operable by keyboard and any pointing device (excluding special cases)?</v>
+      <c r="C26" s="80" t="s">
+        <v>173</v>
       </c>
       <c r="D26" s="32" t="s">
         <v>73</v>
@@ -9847,15 +9830,14 @@
       <c r="G26" s="80"/>
     </row>
     <row r="27" spans="1:64" s="71" customFormat="1" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A27" s="106" t="s">
+      <c r="A27" s="103" t="s">
         <v>92</v>
       </c>
       <c r="B27" s="81">
         <v>8.1</v>
       </c>
-      <c r="C27" s="82" t="str">
-        <f>Criteria!C26</f>
-        <v>Has each web page a defined document type?</v>
+      <c r="C27" s="82" t="s">
+        <v>174</v>
       </c>
       <c r="D27" s="32" t="s">
         <v>73</v>
@@ -9924,14 +9906,13 @@
       <c r="BL27" s="5"/>
     </row>
     <row r="28" spans="1:64" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A28" s="98"/>
+      <c r="A28" s="95"/>
       <c r="B28" s="46" t="str">
         <f>Criteria!B27</f>
         <v>8.2</v>
       </c>
-      <c r="C28" s="32" t="str">
-        <f>Criteria!C27</f>
-        <v>For each web page, is the generated source code valid for the specified document type?</v>
+      <c r="C28" s="32" t="s">
+        <v>143</v>
       </c>
       <c r="D28" s="32" t="s">
         <v>73</v>
@@ -10000,14 +9981,13 @@
       <c r="BL28" s="5"/>
     </row>
     <row r="29" spans="1:64" s="3" customFormat="1" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A29" s="98"/>
+      <c r="A29" s="95"/>
       <c r="B29" s="46" t="str">
         <f>Criteria!B28</f>
         <v>8.3</v>
       </c>
-      <c r="C29" s="32" t="str">
-        <f>Criteria!C28</f>
-        <v>On each web page, is the default language present?</v>
+      <c r="C29" s="32" t="s">
+        <v>144</v>
       </c>
       <c r="D29" s="32" t="s">
         <v>73</v>
@@ -10076,14 +10056,13 @@
       <c r="BL29" s="5"/>
     </row>
     <row r="30" spans="1:64" ht="30" x14ac:dyDescent="0.2">
-      <c r="A30" s="98"/>
+      <c r="A30" s="95"/>
       <c r="B30" s="46" t="str">
         <f>Criteria!B29</f>
         <v>8.4</v>
       </c>
-      <c r="C30" s="32" t="str">
-        <f>Criteria!C29</f>
-        <v>For each web page with a default language, is the language code relevant?</v>
+      <c r="C30" s="32" t="s">
+        <v>145</v>
       </c>
       <c r="D30" s="32" t="s">
         <v>73</v>
@@ -10095,14 +10074,13 @@
       <c r="G30" s="32"/>
     </row>
     <row r="31" spans="1:64" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A31" s="98"/>
+      <c r="A31" s="95"/>
       <c r="B31" s="46" t="str">
         <f>Criteria!B30</f>
         <v>8.5</v>
       </c>
-      <c r="C31" s="32" t="str">
-        <f>Criteria!C30</f>
-        <v>Does every web page have a page title?</v>
+      <c r="C31" s="32" t="s">
+        <v>146</v>
       </c>
       <c r="D31" s="32" t="s">
         <v>73</v>
@@ -10114,14 +10092,13 @@
       <c r="G31" s="32"/>
     </row>
     <row r="32" spans="1:64" ht="30" x14ac:dyDescent="0.2">
-      <c r="A32" s="98"/>
+      <c r="A32" s="95"/>
       <c r="B32" s="46" t="str">
         <f>Criteria!B31</f>
         <v>8.6</v>
       </c>
-      <c r="C32" s="32" t="str">
-        <f>Criteria!C31</f>
-        <v>For each web page with a page title, is this title relevant?</v>
+      <c r="C32" s="32" t="s">
+        <v>147</v>
       </c>
       <c r="D32" s="32" t="s">
         <v>73</v>
@@ -10133,14 +10110,13 @@
       <c r="G32" s="32"/>
     </row>
     <row r="33" spans="1:7" ht="30" x14ac:dyDescent="0.2">
-      <c r="A33" s="98"/>
+      <c r="A33" s="95"/>
       <c r="B33" s="46" t="str">
         <f>Criteria!B32</f>
         <v>8.7</v>
       </c>
-      <c r="C33" s="32" t="str">
-        <f>Criteria!C32</f>
-        <v>On each web page, is each language change indicated in the source code (excluding special cases)?</v>
+      <c r="C33" s="32" t="s">
+        <v>148</v>
       </c>
       <c r="D33" s="32" t="s">
         <v>73</v>
@@ -10152,14 +10128,13 @@
       <c r="G33" s="32"/>
     </row>
     <row r="34" spans="1:7" ht="30" x14ac:dyDescent="0.2">
-      <c r="A34" s="107"/>
+      <c r="A34" s="104"/>
       <c r="B34" s="84" t="str">
         <f>Criteria!B33</f>
         <v>8.8</v>
       </c>
-      <c r="C34" s="85" t="str">
-        <f>Criteria!C33</f>
-        <v>On each web page, is the language code for each language change valid and relevant?</v>
+      <c r="C34" s="85" t="s">
+        <v>149</v>
       </c>
       <c r="D34" s="32" t="s">
         <v>73</v>
@@ -10171,7 +10146,7 @@
       <c r="G34" s="85"/>
     </row>
     <row r="35" spans="1:7" ht="30" x14ac:dyDescent="0.2">
-      <c r="A35" s="103" t="str">
+      <c r="A35" s="105" t="str">
         <f>Criteria!$A$34</f>
         <v>STRUCTURATION</v>
       </c>
@@ -10179,9 +10154,8 @@
         <f>Criteria!B34</f>
         <v>9.1</v>
       </c>
-      <c r="C35" s="82" t="str">
-        <f>Criteria!C34</f>
-        <v>On each web page, is the information structured by the appropriate use of headings?</v>
+      <c r="C35" s="82" t="s">
+        <v>175</v>
       </c>
       <c r="D35" s="32" t="s">
         <v>73</v>
@@ -10193,14 +10167,13 @@
       <c r="G35" s="82"/>
     </row>
     <row r="36" spans="1:7" ht="30" x14ac:dyDescent="0.2">
-      <c r="A36" s="104"/>
+      <c r="A36" s="107"/>
       <c r="B36" s="84" t="str">
         <f>Criteria!B35</f>
         <v>9.2</v>
       </c>
-      <c r="C36" s="85" t="str">
-        <f>Criteria!C35</f>
-        <v>On each web page, is the document structure consistent (excluding special cases)?</v>
+      <c r="C36" s="85" t="s">
+        <v>150</v>
       </c>
       <c r="D36" s="32" t="s">
         <v>73</v>
@@ -10212,16 +10185,15 @@
       <c r="G36" s="85"/>
     </row>
     <row r="37" spans="1:7" ht="30" x14ac:dyDescent="0.2">
-      <c r="A37" s="103" t="s">
+      <c r="A37" s="105" t="s">
         <v>93</v>
       </c>
       <c r="B37" s="81" t="str">
         <f>Criteria!B36</f>
         <v>10.7</v>
       </c>
-      <c r="C37" s="82" t="str">
-        <f>Criteria!C36</f>
-        <v>On each web page, for each element receiving the focus, is the focus visible?</v>
+      <c r="C37" s="82" t="s">
+        <v>151</v>
       </c>
       <c r="D37" s="32" t="s">
         <v>73</v>
@@ -10233,14 +10205,13 @@
       <c r="G37" s="82"/>
     </row>
     <row r="38" spans="1:7" ht="30" x14ac:dyDescent="0.2">
-      <c r="A38" s="105"/>
+      <c r="A38" s="106"/>
       <c r="B38" s="46" t="str">
         <f>Criteria!B37</f>
         <v>10.8</v>
       </c>
-      <c r="C38" s="32" t="str">
-        <f>Criteria!C37</f>
-        <v>For each web page, should hidden content be ignored by assistive technologies?</v>
+      <c r="C38" s="32" t="s">
+        <v>152</v>
       </c>
       <c r="D38" s="32" t="s">
         <v>73</v>
@@ -10252,14 +10223,13 @@
       <c r="G38" s="32"/>
     </row>
     <row r="39" spans="1:7" ht="30" x14ac:dyDescent="0.2">
-      <c r="A39" s="105"/>
+      <c r="A39" s="106"/>
       <c r="B39" s="46" t="str">
         <f>Criteria!B38</f>
         <v>10.9</v>
       </c>
-      <c r="C39" s="32" t="str">
-        <f>Criteria!C38</f>
-        <v>On each web page, information must not be conveyed solely by shape, size or location. Is this rule respected?</v>
+      <c r="C39" s="32" t="s">
+        <v>153</v>
       </c>
       <c r="D39" s="32" t="s">
         <v>73</v>
@@ -10271,14 +10241,13 @@
       <c r="G39" s="32"/>
     </row>
     <row r="40" spans="1:7" ht="45" x14ac:dyDescent="0.2">
-      <c r="A40" s="105"/>
+      <c r="A40" s="106"/>
       <c r="B40" s="46" t="str">
         <f>Criteria!B39</f>
         <v>10.10</v>
       </c>
-      <c r="C40" s="32" t="str">
-        <f>Criteria!C39</f>
-        <v>On each web page, information must not be conveyed by shape, size or location only. Is this rule implemented appropriately?</v>
+      <c r="C40" s="32" t="s">
+        <v>154</v>
       </c>
       <c r="D40" s="32" t="s">
         <v>73</v>
@@ -10290,14 +10259,13 @@
       <c r="G40" s="32"/>
     </row>
     <row r="41" spans="1:7" ht="45" x14ac:dyDescent="0.2">
-      <c r="A41" s="104"/>
+      <c r="A41" s="107"/>
       <c r="B41" s="84" t="str">
         <f>Criteria!B40</f>
         <v>10.14</v>
       </c>
-      <c r="C41" s="85" t="str">
-        <f>Criteria!C40</f>
-        <v>On each web page, can additional content that appears using CSS styles only be made visible using the keyboard and any pointing device?</v>
+      <c r="C41" s="85" t="s">
+        <v>155</v>
       </c>
       <c r="D41" s="32" t="s">
         <v>73</v>
@@ -10309,7 +10277,7 @@
       <c r="G41" s="85"/>
     </row>
     <row r="42" spans="1:7" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A42" s="103" t="str">
+      <c r="A42" s="105" t="str">
         <f>Criteria!$A$41</f>
         <v>FORMS</v>
       </c>
@@ -10317,9 +10285,8 @@
         <f>Criteria!B41</f>
         <v>11.1</v>
       </c>
-      <c r="C42" s="82" t="str">
-        <f>Criteria!C41</f>
-        <v>Does each form input field have a label?</v>
+      <c r="C42" s="82" t="s">
+        <v>156</v>
       </c>
       <c r="D42" s="32" t="s">
         <v>73</v>
@@ -10331,14 +10298,13 @@
       <c r="G42" s="82"/>
     </row>
     <row r="43" spans="1:7" ht="30" x14ac:dyDescent="0.2">
-      <c r="A43" s="105"/>
+      <c r="A43" s="106"/>
       <c r="B43" s="46" t="str">
         <f>Criteria!B42</f>
         <v>11.2</v>
       </c>
-      <c r="C43" s="32" t="str">
-        <f>Criteria!C42</f>
-        <v>Is each label associated with a form field relevant (excluding special cases)?</v>
+      <c r="C43" s="32" t="s">
+        <v>157</v>
       </c>
       <c r="D43" s="32" t="s">
         <v>73</v>
@@ -10350,14 +10316,13 @@
       <c r="G43" s="32"/>
     </row>
     <row r="44" spans="1:7" ht="30" x14ac:dyDescent="0.2">
-      <c r="A44" s="105"/>
+      <c r="A44" s="106"/>
       <c r="B44" s="46" t="str">
         <f>Criteria!B43</f>
         <v>11.5</v>
       </c>
-      <c r="C44" s="32" t="str">
-        <f>Criteria!C43</f>
-        <v>In each form, are the related form controls grouped together, if necessary?</v>
+      <c r="C44" s="32" t="s">
+        <v>176</v>
       </c>
       <c r="D44" s="32" t="s">
         <v>73</v>
@@ -10369,14 +10334,13 @@
       <c r="G44" s="32"/>
     </row>
     <row r="45" spans="1:7" ht="30" x14ac:dyDescent="0.2">
-      <c r="A45" s="105"/>
+      <c r="A45" s="106"/>
       <c r="B45" s="46" t="str">
         <f>Criteria!B44</f>
         <v>11.6</v>
       </c>
-      <c r="C45" s="32" t="str">
-        <f>Criteria!C44</f>
-        <v>In each form, does each group of related form controls have a legend?</v>
+      <c r="C45" s="32" t="s">
+        <v>177</v>
       </c>
       <c r="D45" s="32" t="s">
         <v>73</v>
@@ -10388,14 +10352,13 @@
       <c r="G45" s="32"/>
     </row>
     <row r="46" spans="1:7" ht="30" x14ac:dyDescent="0.2">
-      <c r="A46" s="105"/>
+      <c r="A46" s="106"/>
       <c r="B46" s="46" t="str">
         <f>Criteria!B45</f>
         <v>11.7</v>
       </c>
-      <c r="C46" s="32" t="str">
-        <f>Criteria!C45</f>
-        <v>In each form, is each legend associated with a group of related form controls relevant?</v>
+      <c r="C46" s="32" t="s">
+        <v>178</v>
       </c>
       <c r="D46" s="32" t="s">
         <v>73</v>
@@ -10407,14 +10370,13 @@
       <c r="G46" s="32"/>
     </row>
     <row r="47" spans="1:7" ht="30" x14ac:dyDescent="0.2">
-      <c r="A47" s="105"/>
+      <c r="A47" s="106"/>
       <c r="B47" s="46" t="str">
         <f>Criteria!B46</f>
         <v>11.9</v>
       </c>
-      <c r="C47" s="32" t="str">
-        <f>Criteria!C46</f>
-        <v>In each form, is the label of each button relevant (excluding special cases)?</v>
+      <c r="C47" s="32" t="s">
+        <v>179</v>
       </c>
       <c r="D47" s="32" t="s">
         <v>73</v>
@@ -10426,14 +10388,13 @@
       <c r="G47" s="32"/>
     </row>
     <row r="48" spans="1:7" ht="30" x14ac:dyDescent="0.2">
-      <c r="A48" s="104"/>
+      <c r="A48" s="107"/>
       <c r="B48" s="84" t="str">
         <f>Criteria!B47</f>
         <v>11.10</v>
       </c>
-      <c r="C48" s="85" t="str">
-        <f>Criteria!C47</f>
-        <v>In each form, is the error management used appropriately (excluding special cases)?</v>
+      <c r="C48" s="85" t="s">
+        <v>185</v>
       </c>
       <c r="D48" s="32" t="s">
         <v>73</v>
@@ -10445,16 +10406,15 @@
       <c r="G48" s="85"/>
     </row>
     <row r="49" spans="1:7" ht="45" x14ac:dyDescent="0.2">
-      <c r="A49" s="103" t="s">
+      <c r="A49" s="105" t="s">
         <v>57</v>
       </c>
       <c r="B49" s="81" t="str">
         <f>Criteria!B48</f>
         <v>12.6</v>
       </c>
-      <c r="C49" s="82" t="str">
-        <f>Criteria!C48</f>
-        <v>Can content grouping regions present in several web pages header, main navigation, main content, footer and search engine) be reached or avoided?</v>
+      <c r="C49" s="82" t="s">
+        <v>186</v>
       </c>
       <c r="D49" s="32" t="s">
         <v>73</v>
@@ -10466,14 +10426,13 @@
       <c r="G49" s="82"/>
     </row>
     <row r="50" spans="1:7" ht="30" x14ac:dyDescent="0.2">
-      <c r="A50" s="105"/>
+      <c r="A50" s="106"/>
       <c r="B50" s="46" t="str">
         <f>Criteria!B49</f>
         <v>12.7</v>
       </c>
-      <c r="C50" s="32" t="str">
-        <f>Criteria!C49</f>
-        <v>On each web page, is there a bypass or skip link to the main content region (excluding special cases)?</v>
+      <c r="C50" s="32" t="s">
+        <v>158</v>
       </c>
       <c r="D50" s="32" t="s">
         <v>73</v>
@@ -10485,14 +10444,13 @@
       <c r="G50" s="32"/>
     </row>
     <row r="51" spans="1:7" ht="30" x14ac:dyDescent="0.2">
-      <c r="A51" s="105"/>
+      <c r="A51" s="106"/>
       <c r="B51" s="46" t="str">
         <f>Criteria!B50</f>
         <v>12.8</v>
       </c>
-      <c r="C51" s="32" t="str">
-        <f>Criteria!C50</f>
-        <v>On each web page, is the navigation sequence consistent?</v>
+      <c r="C51" s="32" t="s">
+        <v>182</v>
       </c>
       <c r="D51" s="32" t="s">
         <v>73</v>
@@ -10504,14 +10462,13 @@
       <c r="G51" s="32"/>
     </row>
     <row r="52" spans="1:7" ht="30" x14ac:dyDescent="0.2">
-      <c r="A52" s="105"/>
+      <c r="A52" s="106"/>
       <c r="B52" s="46" t="str">
         <f>Criteria!B51</f>
         <v>12.9</v>
       </c>
-      <c r="C52" s="32" t="str">
-        <f>Criteria!C51</f>
-        <v>On each web page, navigation must not contain any keyboard traps. Is this rule respected?</v>
+      <c r="C52" s="32" t="s">
+        <v>159</v>
       </c>
       <c r="D52" s="32" t="s">
         <v>73</v>
@@ -10523,14 +10480,13 @@
       <c r="G52" s="32"/>
     </row>
     <row r="53" spans="1:7" ht="60" x14ac:dyDescent="0.2">
-      <c r="A53" s="104"/>
+      <c r="A53" s="107"/>
       <c r="B53" s="84" t="str">
         <f>Criteria!B52</f>
         <v>12.11</v>
       </c>
-      <c r="C53" s="85" t="str">
-        <f>Criteria!C52</f>
-        <v>On each web page, is the additional content that appears when hovering over, focusing on or activating a user interface component accessible by keyboard if necessary?</v>
+      <c r="C53" s="85" t="s">
+        <v>160</v>
       </c>
       <c r="D53" s="32" t="s">
         <v>73</v>
@@ -10542,7 +10498,7 @@
       <c r="G53" s="85"/>
     </row>
     <row r="54" spans="1:7" ht="45" x14ac:dyDescent="0.2">
-      <c r="A54" s="103" t="str">
+      <c r="A54" s="105" t="str">
         <f>Criteria!$A$53</f>
         <v>CONSULTATION</v>
       </c>
@@ -10550,9 +10506,8 @@
         <f>Criteria!B53</f>
         <v>13.1</v>
       </c>
-      <c r="C54" s="82" t="str">
-        <f>Criteria!C53</f>
-        <v>For each web page, does the user have control over each time limit for modifying the content (excluding special cases)?</v>
+      <c r="C54" s="82" t="s">
+        <v>161</v>
       </c>
       <c r="D54" s="32" t="s">
         <v>73</v>
@@ -10564,14 +10519,13 @@
       <c r="G54" s="82"/>
     </row>
     <row r="55" spans="1:7" ht="30" x14ac:dyDescent="0.2">
-      <c r="A55" s="105"/>
+      <c r="A55" s="106"/>
       <c r="B55" s="46" t="str">
         <f>Criteria!B54</f>
         <v>13.7</v>
       </c>
-      <c r="C55" s="32" t="str">
-        <f>Criteria!C54</f>
-        <v>On each web page, are sudden changes in brightness or blinking used correctly?</v>
+      <c r="C55" s="32" t="s">
+        <v>183</v>
       </c>
       <c r="D55" s="32" t="s">
         <v>73</v>
@@ -10583,14 +10537,13 @@
       <c r="G55" s="32"/>
     </row>
     <row r="56" spans="1:7" ht="30" x14ac:dyDescent="0.2">
-      <c r="A56" s="104"/>
+      <c r="A56" s="107"/>
       <c r="B56" s="84" t="str">
         <f>Criteria!B55</f>
         <v>13.8</v>
       </c>
-      <c r="C56" s="85" t="str">
-        <f>Criteria!C55</f>
-        <v>On each web page, is every moving or blinking content controllable by the user?</v>
+      <c r="C56" s="85" t="s">
+        <v>184</v>
       </c>
       <c r="D56" s="32" t="s">
         <v>73</v>
@@ -10603,6 +10556,11 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="A37:A41"/>
+    <mergeCell ref="A42:A48"/>
+    <mergeCell ref="A49:A53"/>
+    <mergeCell ref="A54:A56"/>
     <mergeCell ref="A27:A34"/>
     <mergeCell ref="A14:A21"/>
     <mergeCell ref="A22:A23"/>
@@ -10611,11 +10569,6 @@
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A4:A10"/>
     <mergeCell ref="A12:A13"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="A37:A41"/>
-    <mergeCell ref="A42:A48"/>
-    <mergeCell ref="A49:A53"/>
-    <mergeCell ref="A54:A56"/>
   </mergeCells>
   <conditionalFormatting sqref="D4:D56">
     <cfRule type="cellIs" dxfId="17" priority="8" operator="equal">
@@ -10778,7 +10731,7 @@
       <c r="BL3" s="48"/>
     </row>
     <row r="4" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A4" s="103" t="str">
+      <c r="A4" s="105" t="str">
         <f>Criteria!$A$3</f>
         <v>IMAGES</v>
       </c>
@@ -10786,9 +10739,8 @@
         <f>Criteria!B3</f>
         <v>1.1</v>
       </c>
-      <c r="C4" s="82" t="str">
-        <f>Criteria!C3</f>
-        <v>Does each image conveying information have a text alternative?</v>
+      <c r="C4" s="32" t="s">
+        <v>125</v>
       </c>
       <c r="D4" s="32" t="s">
         <v>73</v>
@@ -10856,14 +10808,13 @@
       <c r="BL4" s="48"/>
     </row>
     <row r="5" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A5" s="105"/>
+      <c r="A5" s="106"/>
       <c r="B5" s="46" t="str">
         <f>Criteria!B4</f>
         <v>1.2</v>
       </c>
-      <c r="C5" s="32" t="str">
-        <f>Criteria!C4</f>
-        <v>Is every decorative image correctly ignored by assistive technologies?</v>
+      <c r="C5" s="32" t="s">
+        <v>126</v>
       </c>
       <c r="D5" s="32" t="s">
         <v>73</v>
@@ -10932,14 +10883,13 @@
       <c r="BL5" s="48"/>
     </row>
     <row r="6" spans="1:64" s="49" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A6" s="105"/>
+      <c r="A6" s="106"/>
       <c r="B6" s="46" t="str">
         <f>Criteria!B5</f>
         <v>1.3</v>
       </c>
-      <c r="C6" s="32" t="str">
-        <f>Criteria!C5</f>
-        <v>For each image conveying information with a text alternative, is this alternative relevant (excluding special cases)?</v>
+      <c r="C6" s="32" t="s">
+        <v>127</v>
       </c>
       <c r="D6" s="32" t="s">
         <v>73</v>
@@ -11008,14 +10958,13 @@
       <c r="BL6" s="48"/>
     </row>
     <row r="7" spans="1:64" s="49" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A7" s="105"/>
+      <c r="A7" s="106"/>
       <c r="B7" s="46" t="str">
         <f>Criteria!B6</f>
         <v>1.4</v>
       </c>
-      <c r="C7" s="32" t="str">
-        <f>Criteria!C6</f>
-        <v>For each image used as a CAPTCHA or test image, with a text alternative, does this alternative make it possible to identify the nature and function of the image?</v>
+      <c r="C7" s="32" t="s">
+        <v>128</v>
       </c>
       <c r="D7" s="32" t="s">
         <v>73</v>
@@ -11084,14 +11033,13 @@
       <c r="BL7" s="48"/>
     </row>
     <row r="8" spans="1:64" s="49" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A8" s="105"/>
+      <c r="A8" s="106"/>
       <c r="B8" s="46" t="str">
         <f>Criteria!B7</f>
         <v>1.5</v>
       </c>
-      <c r="C8" s="32" t="str">
-        <f>Criteria!C7</f>
-        <v>For each image used as a CAPTCHA, is there an alternative access solution to the content or to the CAPTCHA function?</v>
+      <c r="C8" s="32" t="s">
+        <v>129</v>
       </c>
       <c r="D8" s="32" t="s">
         <v>73</v>
@@ -11160,14 +11108,13 @@
       <c r="BL8" s="48"/>
     </row>
     <row r="9" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A9" s="105"/>
+      <c r="A9" s="106"/>
       <c r="B9" s="46" t="str">
         <f>Criteria!B8</f>
         <v>1.6</v>
       </c>
-      <c r="C9" s="32" t="str">
-        <f>Criteria!C8</f>
-        <v>Does each image conveying information have, if necessary, a detailed description?</v>
+      <c r="C9" s="32" t="s">
+        <v>130</v>
       </c>
       <c r="D9" s="32" t="s">
         <v>73</v>
@@ -11236,14 +11183,13 @@
       <c r="BL9" s="48"/>
     </row>
     <row r="10" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A10" s="104"/>
+      <c r="A10" s="107"/>
       <c r="B10" s="84" t="str">
         <f>Criteria!B9</f>
         <v>1.7</v>
       </c>
-      <c r="C10" s="85" t="str">
-        <f>Criteria!C9</f>
-        <v>For each image conveying information with a detailed description, is this description relevant?</v>
+      <c r="C10" s="75" t="s">
+        <v>131</v>
       </c>
       <c r="D10" s="32" t="s">
         <v>73</v>
@@ -11320,9 +11266,8 @@
         <f>Criteria!B10</f>
         <v>2.1</v>
       </c>
-      <c r="C11" s="80" t="str">
-        <f>Criteria!C10</f>
-        <v>Does each frame have a frame title?</v>
+      <c r="C11" s="80" t="s">
+        <v>132</v>
       </c>
       <c r="D11" s="32" t="s">
         <v>73</v>
@@ -11391,7 +11336,7 @@
       <c r="BL11" s="48"/>
     </row>
     <row r="12" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A12" s="103" t="str">
+      <c r="A12" s="105" t="str">
         <f>Criteria!$A$11</f>
         <v>COLOURS</v>
       </c>
@@ -11399,9 +11344,8 @@
         <f>Criteria!B11</f>
         <v>3.1</v>
       </c>
-      <c r="C12" s="82" t="str">
-        <f>Criteria!C11</f>
-        <v>On each web page, the information must not be provided by colour alone. Is this rule respected?</v>
+      <c r="C12" s="77" t="s">
+        <v>169</v>
       </c>
       <c r="D12" s="32" t="s">
         <v>73</v>
@@ -11470,14 +11414,13 @@
       <c r="BL12" s="48"/>
     </row>
     <row r="13" spans="1:64" s="49" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A13" s="104"/>
+      <c r="A13" s="107"/>
       <c r="B13" s="84" t="str">
         <f>Criteria!B12</f>
         <v>3.2</v>
       </c>
-      <c r="C13" s="85" t="str">
-        <f>Criteria!C12</f>
-        <v>On each web page, is the contrast between the colour of the text and the colour of its background sufficiently high (excluding special cases)?</v>
+      <c r="C13" s="75" t="s">
+        <v>133</v>
       </c>
       <c r="D13" s="32" t="s">
         <v>73</v>
@@ -11546,7 +11489,7 @@
       <c r="BL13" s="48"/>
     </row>
     <row r="14" spans="1:64" s="49" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A14" s="103" t="str">
+      <c r="A14" s="105" t="str">
         <f>Criteria!$A$13</f>
         <v>MULTIMEDIA</v>
       </c>
@@ -11554,9 +11497,8 @@
         <f>Criteria!B13</f>
         <v>4.1</v>
       </c>
-      <c r="C14" s="82" t="str">
-        <f>Criteria!C13</f>
-        <v>Does each pre-recorded time-based media have, if necessary, a transcript or an audio description (excluding special cases)?</v>
+      <c r="C14" s="82" t="s">
+        <v>134</v>
       </c>
       <c r="D14" s="32" t="s">
         <v>73</v>
@@ -11625,14 +11567,13 @@
       <c r="BL14" s="48"/>
     </row>
     <row r="15" spans="1:64" s="49" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A15" s="105"/>
+      <c r="A15" s="106"/>
       <c r="B15" s="46" t="str">
         <f>Criteria!B14</f>
         <v>4.2</v>
       </c>
-      <c r="C15" s="32" t="str">
-        <f>Criteria!C14</f>
-        <v>For each pre-recorded time-based media with a synchronised transcript or audio description, are these relevant (excluding special cases)?</v>
+      <c r="C15" s="32" t="s">
+        <v>135</v>
       </c>
       <c r="D15" s="32" t="s">
         <v>73</v>
@@ -11701,14 +11642,13 @@
       <c r="BL15" s="48"/>
     </row>
     <row r="16" spans="1:64" s="49" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A16" s="105"/>
+      <c r="A16" s="106"/>
       <c r="B16" s="46" t="str">
         <f>Criteria!B15</f>
         <v>4.3</v>
       </c>
-      <c r="C16" s="32" t="str">
-        <f>Criteria!C15</f>
-        <v>Does each pre-recorded synchronised time-based media have, if necessary, synchronised captions (excluding special cases)?</v>
+      <c r="C16" s="32" t="s">
+        <v>170</v>
       </c>
       <c r="D16" s="32" t="s">
         <v>73</v>
@@ -11777,14 +11717,13 @@
       <c r="BL16" s="48"/>
     </row>
     <row r="17" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A17" s="105"/>
+      <c r="A17" s="106"/>
       <c r="B17" s="46" t="str">
         <f>Criteria!B16</f>
         <v>4.4</v>
       </c>
-      <c r="C17" s="32" t="str">
-        <f>Criteria!C16</f>
-        <v>For each pre-recorded synchronised time-based media with synchronised subtitles, are these captions relevant?</v>
+      <c r="C17" s="32" t="s">
+        <v>171</v>
       </c>
       <c r="D17" s="32" t="s">
         <v>73</v>
@@ -11853,14 +11792,13 @@
       <c r="BL17" s="48"/>
     </row>
     <row r="18" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A18" s="105"/>
+      <c r="A18" s="106"/>
       <c r="B18" s="46" t="str">
         <f>Criteria!B17</f>
         <v>4.8</v>
       </c>
-      <c r="C18" s="32" t="str">
-        <f>Criteria!C17</f>
-        <v>Does each non-time-based media have, if necessary, an alternative (excluding special cases)?</v>
+      <c r="C18" s="32" t="s">
+        <v>136</v>
       </c>
       <c r="D18" s="32" t="s">
         <v>73</v>
@@ -11929,14 +11867,13 @@
       <c r="BL18" s="48"/>
     </row>
     <row r="19" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A19" s="105"/>
+      <c r="A19" s="106"/>
       <c r="B19" s="46" t="str">
         <f>Criteria!B18</f>
         <v>4.9</v>
       </c>
-      <c r="C19" s="32" t="str">
-        <f>Criteria!C18</f>
-        <v>For each non-time-based media having an alternative, is this alternative relevant?</v>
+      <c r="C19" s="32" t="s">
+        <v>137</v>
       </c>
       <c r="D19" s="32" t="s">
         <v>73</v>
@@ -12005,14 +11942,13 @@
       <c r="BL19" s="48"/>
     </row>
     <row r="20" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A20" s="105"/>
+      <c r="A20" s="106"/>
       <c r="B20" s="46" t="str">
         <f>Criteria!B19</f>
         <v>4.10</v>
       </c>
-      <c r="C20" s="32" t="str">
-        <f>Criteria!C19</f>
-        <v>Is each automatically triggered sound controllable by the user?</v>
+      <c r="C20" s="32" t="s">
+        <v>138</v>
       </c>
       <c r="D20" s="32" t="s">
         <v>73</v>
@@ -12081,14 +12017,13 @@
       <c r="BL20" s="48"/>
     </row>
     <row r="21" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A21" s="104"/>
+      <c r="A21" s="107"/>
       <c r="B21" s="84" t="str">
         <f>Criteria!B20</f>
         <v>4.11</v>
       </c>
-      <c r="C21" s="85" t="str">
-        <f>Criteria!C20</f>
-        <v>Is the viewing of each time-based media, if required, controllable by keyboard and any pointing device?</v>
+      <c r="C21" s="85" t="s">
+        <v>139</v>
       </c>
       <c r="D21" s="32" t="s">
         <v>73</v>
@@ -12157,16 +12092,15 @@
       <c r="BL21" s="48"/>
     </row>
     <row r="22" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A22" s="103" t="s">
+      <c r="A22" s="105" t="s">
         <v>26</v>
       </c>
       <c r="B22" s="81" t="str">
         <f>Criteria!B21</f>
         <v>5.6</v>
       </c>
-      <c r="C22" s="82" t="str">
-        <f>Criteria!C21</f>
-        <v>For each data table, are each column header and each row header correctly declared?</v>
+      <c r="C22" s="82" t="s">
+        <v>140</v>
       </c>
       <c r="D22" s="32" t="s">
         <v>73</v>
@@ -12235,14 +12169,13 @@
       <c r="BL22" s="48"/>
     </row>
     <row r="23" spans="1:64" s="49" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A23" s="104"/>
+      <c r="A23" s="107"/>
       <c r="B23" s="84" t="str">
         <f>Criteria!B22</f>
         <v>5.7</v>
       </c>
-      <c r="C23" s="85" t="str">
-        <f>Criteria!C22</f>
-        <v>For each data table, is the appropriate technique used to associate each cell with its headers (excluding special cases)?</v>
+      <c r="C23" s="85" t="s">
+        <v>141</v>
       </c>
       <c r="D23" s="32" t="s">
         <v>73</v>
@@ -12311,7 +12244,7 @@
       <c r="BL23" s="48"/>
     </row>
     <row r="24" spans="1:64" s="49" customFormat="1" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A24" s="103" t="str">
+      <c r="A24" s="105" t="str">
         <f>Criteria!$A$23</f>
         <v>LINKS</v>
       </c>
@@ -12319,9 +12252,8 @@
         <f>Criteria!B23</f>
         <v>6.1</v>
       </c>
-      <c r="C24" s="82" t="str">
-        <f>Criteria!C23</f>
-        <v>Is every link explicit (except in special cases)?</v>
+      <c r="C24" s="82" t="s">
+        <v>142</v>
       </c>
       <c r="D24" s="32" t="s">
         <v>73</v>
@@ -12390,14 +12322,13 @@
       <c r="BL24" s="48"/>
     </row>
     <row r="25" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A25" s="104"/>
+      <c r="A25" s="107"/>
       <c r="B25" s="84" t="str">
         <f>Criteria!B24</f>
         <v>6.2</v>
       </c>
-      <c r="C25" s="85" t="str">
-        <f>Criteria!C24</f>
-        <v>On each web page, does each link have an accessible name?</v>
+      <c r="C25" s="85" t="s">
+        <v>172</v>
       </c>
       <c r="D25" s="32" t="s">
         <v>73</v>
@@ -12473,9 +12404,8 @@
         <f>Criteria!B25</f>
         <v>7.3</v>
       </c>
-      <c r="C26" s="80" t="str">
-        <f>Criteria!C25</f>
-        <v>Is each script accessible and operable by keyboard and any pointing device (excluding special cases)?</v>
+      <c r="C26" s="80" t="s">
+        <v>173</v>
       </c>
       <c r="D26" s="32" t="s">
         <v>73</v>
@@ -12544,15 +12474,14 @@
       <c r="BL26" s="48"/>
     </row>
     <row r="27" spans="1:64" s="49" customFormat="1" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A27" s="106" t="s">
+      <c r="A27" s="103" t="s">
         <v>92</v>
       </c>
       <c r="B27" s="81">
         <v>8.1</v>
       </c>
-      <c r="C27" s="82" t="str">
-        <f>Criteria!C26</f>
-        <v>Has each web page a defined document type?</v>
+      <c r="C27" s="82" t="s">
+        <v>174</v>
       </c>
       <c r="D27" s="32" t="s">
         <v>73</v>
@@ -12621,14 +12550,13 @@
       <c r="BL27" s="48"/>
     </row>
     <row r="28" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A28" s="98"/>
+      <c r="A28" s="95"/>
       <c r="B28" s="46" t="str">
         <f>Criteria!B27</f>
         <v>8.2</v>
       </c>
-      <c r="C28" s="32" t="str">
-        <f>Criteria!C27</f>
-        <v>For each web page, is the generated source code valid for the specified document type?</v>
+      <c r="C28" s="32" t="s">
+        <v>143</v>
       </c>
       <c r="D28" s="32" t="s">
         <v>73</v>
@@ -12697,14 +12625,13 @@
       <c r="BL28" s="48"/>
     </row>
     <row r="29" spans="1:64" s="49" customFormat="1" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A29" s="98"/>
+      <c r="A29" s="95"/>
       <c r="B29" s="46" t="str">
         <f>Criteria!B28</f>
         <v>8.3</v>
       </c>
-      <c r="C29" s="32" t="str">
-        <f>Criteria!C28</f>
-        <v>On each web page, is the default language present?</v>
+      <c r="C29" s="32" t="s">
+        <v>144</v>
       </c>
       <c r="D29" s="32" t="s">
         <v>73</v>
@@ -12773,14 +12700,13 @@
       <c r="BL29" s="48"/>
     </row>
     <row r="30" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A30" s="98"/>
+      <c r="A30" s="95"/>
       <c r="B30" s="46" t="str">
         <f>Criteria!B29</f>
         <v>8.4</v>
       </c>
-      <c r="C30" s="32" t="str">
-        <f>Criteria!C29</f>
-        <v>For each web page with a default language, is the language code relevant?</v>
+      <c r="C30" s="32" t="s">
+        <v>145</v>
       </c>
       <c r="D30" s="32" t="s">
         <v>73</v>
@@ -12849,14 +12775,13 @@
       <c r="BL30" s="48"/>
     </row>
     <row r="31" spans="1:64" s="49" customFormat="1" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A31" s="98"/>
+      <c r="A31" s="95"/>
       <c r="B31" s="46" t="str">
         <f>Criteria!B30</f>
         <v>8.5</v>
       </c>
-      <c r="C31" s="32" t="str">
-        <f>Criteria!C30</f>
-        <v>Does every web page have a page title?</v>
+      <c r="C31" s="32" t="s">
+        <v>146</v>
       </c>
       <c r="D31" s="32" t="s">
         <v>73</v>
@@ -12925,14 +12850,13 @@
       <c r="BL31" s="48"/>
     </row>
     <row r="32" spans="1:64" s="49" customFormat="1" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A32" s="98"/>
+      <c r="A32" s="95"/>
       <c r="B32" s="46" t="str">
         <f>Criteria!B31</f>
         <v>8.6</v>
       </c>
-      <c r="C32" s="32" t="str">
-        <f>Criteria!C31</f>
-        <v>For each web page with a page title, is this title relevant?</v>
+      <c r="C32" s="32" t="s">
+        <v>147</v>
       </c>
       <c r="D32" s="32" t="s">
         <v>73</v>
@@ -13001,14 +12925,13 @@
       <c r="BL32" s="48"/>
     </row>
     <row r="33" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A33" s="98"/>
+      <c r="A33" s="95"/>
       <c r="B33" s="46" t="str">
         <f>Criteria!B32</f>
         <v>8.7</v>
       </c>
-      <c r="C33" s="32" t="str">
-        <f>Criteria!C32</f>
-        <v>On each web page, is each language change indicated in the source code (excluding special cases)?</v>
+      <c r="C33" s="32" t="s">
+        <v>148</v>
       </c>
       <c r="D33" s="32" t="s">
         <v>73</v>
@@ -13077,14 +13000,13 @@
       <c r="BL33" s="48"/>
     </row>
     <row r="34" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A34" s="98"/>
+      <c r="A34" s="95"/>
       <c r="B34" s="74" t="str">
         <f>Criteria!B33</f>
         <v>8.8</v>
       </c>
-      <c r="C34" s="75" t="str">
-        <f>Criteria!C33</f>
-        <v>On each web page, is the language code for each language change valid and relevant?</v>
+      <c r="C34" s="85" t="s">
+        <v>149</v>
       </c>
       <c r="D34" s="32" t="s">
         <v>73</v>
@@ -13153,7 +13075,7 @@
       <c r="BL34" s="48"/>
     </row>
     <row r="35" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A35" s="103" t="str">
+      <c r="A35" s="105" t="str">
         <f>Criteria!$A$34</f>
         <v>STRUCTURATION</v>
       </c>
@@ -13161,9 +13083,8 @@
         <f>Criteria!B34</f>
         <v>9.1</v>
       </c>
-      <c r="C35" s="82" t="str">
-        <f>Criteria!C34</f>
-        <v>On each web page, is the information structured by the appropriate use of headings?</v>
+      <c r="C35" s="82" t="s">
+        <v>175</v>
       </c>
       <c r="D35" s="32" t="s">
         <v>73</v>
@@ -13232,14 +13153,13 @@
       <c r="BL35" s="48"/>
     </row>
     <row r="36" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A36" s="104"/>
+      <c r="A36" s="107"/>
       <c r="B36" s="84" t="str">
         <f>Criteria!B35</f>
         <v>9.2</v>
       </c>
-      <c r="C36" s="85" t="str">
-        <f>Criteria!C35</f>
-        <v>On each web page, is the document structure consistent (excluding special cases)?</v>
+      <c r="C36" s="85" t="s">
+        <v>150</v>
       </c>
       <c r="D36" s="32" t="s">
         <v>73</v>
@@ -13308,16 +13228,15 @@
       <c r="BL36" s="48"/>
     </row>
     <row r="37" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A37" s="103" t="s">
+      <c r="A37" s="105" t="s">
         <v>93</v>
       </c>
       <c r="B37" s="81" t="str">
         <f>Criteria!B36</f>
         <v>10.7</v>
       </c>
-      <c r="C37" s="82" t="str">
-        <f>Criteria!C36</f>
-        <v>On each web page, for each element receiving the focus, is the focus visible?</v>
+      <c r="C37" s="82" t="s">
+        <v>151</v>
       </c>
       <c r="D37" s="32" t="s">
         <v>73</v>
@@ -13386,14 +13305,13 @@
       <c r="BL37" s="48"/>
     </row>
     <row r="38" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A38" s="105"/>
+      <c r="A38" s="106"/>
       <c r="B38" s="46" t="str">
         <f>Criteria!B37</f>
         <v>10.8</v>
       </c>
-      <c r="C38" s="32" t="str">
-        <f>Criteria!C37</f>
-        <v>For each web page, should hidden content be ignored by assistive technologies?</v>
+      <c r="C38" s="32" t="s">
+        <v>152</v>
       </c>
       <c r="D38" s="32" t="s">
         <v>73</v>
@@ -13462,14 +13380,13 @@
       <c r="BL38" s="48"/>
     </row>
     <row r="39" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A39" s="105"/>
+      <c r="A39" s="106"/>
       <c r="B39" s="46" t="str">
         <f>Criteria!B38</f>
         <v>10.9</v>
       </c>
-      <c r="C39" s="32" t="str">
-        <f>Criteria!C38</f>
-        <v>On each web page, information must not be conveyed solely by shape, size or location. Is this rule respected?</v>
+      <c r="C39" s="32" t="s">
+        <v>153</v>
       </c>
       <c r="D39" s="32" t="s">
         <v>73</v>
@@ -13538,14 +13455,13 @@
       <c r="BL39" s="48"/>
     </row>
     <row r="40" spans="1:64" s="49" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A40" s="105"/>
+      <c r="A40" s="106"/>
       <c r="B40" s="46" t="str">
         <f>Criteria!B39</f>
         <v>10.10</v>
       </c>
-      <c r="C40" s="32" t="str">
-        <f>Criteria!C39</f>
-        <v>On each web page, information must not be conveyed by shape, size or location only. Is this rule implemented appropriately?</v>
+      <c r="C40" s="32" t="s">
+        <v>154</v>
       </c>
       <c r="D40" s="32" t="s">
         <v>73</v>
@@ -13614,14 +13530,13 @@
       <c r="BL40" s="48"/>
     </row>
     <row r="41" spans="1:64" s="49" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A41" s="104"/>
+      <c r="A41" s="107"/>
       <c r="B41" s="84" t="str">
         <f>Criteria!B40</f>
         <v>10.14</v>
       </c>
-      <c r="C41" s="85" t="str">
-        <f>Criteria!C40</f>
-        <v>On each web page, can additional content that appears using CSS styles only be made visible using the keyboard and any pointing device?</v>
+      <c r="C41" s="85" t="s">
+        <v>155</v>
       </c>
       <c r="D41" s="32" t="s">
         <v>73</v>
@@ -13690,7 +13605,7 @@
       <c r="BL41" s="48"/>
     </row>
     <row r="42" spans="1:64" s="49" customFormat="1" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A42" s="103" t="str">
+      <c r="A42" s="105" t="str">
         <f>Criteria!$A$41</f>
         <v>FORMS</v>
       </c>
@@ -13698,9 +13613,8 @@
         <f>Criteria!B41</f>
         <v>11.1</v>
       </c>
-      <c r="C42" s="82" t="str">
-        <f>Criteria!C41</f>
-        <v>Does each form input field have a label?</v>
+      <c r="C42" s="82" t="s">
+        <v>156</v>
       </c>
       <c r="D42" s="32" t="s">
         <v>73</v>
@@ -13769,14 +13683,13 @@
       <c r="BL42" s="48"/>
     </row>
     <row r="43" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A43" s="105"/>
+      <c r="A43" s="106"/>
       <c r="B43" s="46" t="str">
         <f>Criteria!B42</f>
         <v>11.2</v>
       </c>
-      <c r="C43" s="32" t="str">
-        <f>Criteria!C42</f>
-        <v>Is each label associated with a form field relevant (excluding special cases)?</v>
+      <c r="C43" s="32" t="s">
+        <v>157</v>
       </c>
       <c r="D43" s="32" t="s">
         <v>73</v>
@@ -13845,14 +13758,13 @@
       <c r="BL43" s="48"/>
     </row>
     <row r="44" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A44" s="105"/>
+      <c r="A44" s="106"/>
       <c r="B44" s="46" t="str">
         <f>Criteria!B43</f>
         <v>11.5</v>
       </c>
-      <c r="C44" s="32" t="str">
-        <f>Criteria!C43</f>
-        <v>In each form, are the related form controls grouped together, if necessary?</v>
+      <c r="C44" s="32" t="s">
+        <v>176</v>
       </c>
       <c r="D44" s="32" t="s">
         <v>73</v>
@@ -13921,14 +13833,13 @@
       <c r="BL44" s="48"/>
     </row>
     <row r="45" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A45" s="105"/>
+      <c r="A45" s="106"/>
       <c r="B45" s="46" t="str">
         <f>Criteria!B44</f>
         <v>11.6</v>
       </c>
-      <c r="C45" s="32" t="str">
-        <f>Criteria!C44</f>
-        <v>In each form, does each group of related form controls have a legend?</v>
+      <c r="C45" s="32" t="s">
+        <v>177</v>
       </c>
       <c r="D45" s="32" t="s">
         <v>73</v>
@@ -13997,14 +13908,13 @@
       <c r="BL45" s="48"/>
     </row>
     <row r="46" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A46" s="105"/>
+      <c r="A46" s="106"/>
       <c r="B46" s="46" t="str">
         <f>Criteria!B45</f>
         <v>11.7</v>
       </c>
-      <c r="C46" s="32" t="str">
-        <f>Criteria!C45</f>
-        <v>In each form, is each legend associated with a group of related form controls relevant?</v>
+      <c r="C46" s="32" t="s">
+        <v>178</v>
       </c>
       <c r="D46" s="32" t="s">
         <v>73</v>
@@ -14073,14 +13983,13 @@
       <c r="BL46" s="48"/>
     </row>
     <row r="47" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A47" s="105"/>
+      <c r="A47" s="106"/>
       <c r="B47" s="46" t="str">
         <f>Criteria!B46</f>
         <v>11.9</v>
       </c>
-      <c r="C47" s="32" t="str">
-        <f>Criteria!C46</f>
-        <v>In each form, is the label of each button relevant (excluding special cases)?</v>
+      <c r="C47" s="32" t="s">
+        <v>179</v>
       </c>
       <c r="D47" s="32" t="s">
         <v>73</v>
@@ -14149,14 +14058,13 @@
       <c r="BL47" s="48"/>
     </row>
     <row r="48" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A48" s="104"/>
+      <c r="A48" s="107"/>
       <c r="B48" s="84" t="str">
         <f>Criteria!B47</f>
         <v>11.10</v>
       </c>
-      <c r="C48" s="85" t="str">
-        <f>Criteria!C47</f>
-        <v>In each form, is the error management used appropriately (excluding special cases)?</v>
+      <c r="C48" s="85" t="s">
+        <v>185</v>
       </c>
       <c r="D48" s="32" t="s">
         <v>73</v>
@@ -14225,16 +14133,15 @@
       <c r="BL48" s="48"/>
     </row>
     <row r="49" spans="1:64" s="49" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A49" s="103" t="s">
+      <c r="A49" s="105" t="s">
         <v>57</v>
       </c>
       <c r="B49" s="81" t="str">
         <f>Criteria!B48</f>
         <v>12.6</v>
       </c>
-      <c r="C49" s="82" t="str">
-        <f>Criteria!C48</f>
-        <v>Can content grouping regions present in several web pages header, main navigation, main content, footer and search engine) be reached or avoided?</v>
+      <c r="C49" s="82" t="s">
+        <v>186</v>
       </c>
       <c r="D49" s="32" t="s">
         <v>73</v>
@@ -14303,14 +14210,13 @@
       <c r="BL49" s="48"/>
     </row>
     <row r="50" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A50" s="105"/>
+      <c r="A50" s="106"/>
       <c r="B50" s="46" t="str">
         <f>Criteria!B49</f>
         <v>12.7</v>
       </c>
-      <c r="C50" s="32" t="str">
-        <f>Criteria!C49</f>
-        <v>On each web page, is there a bypass or skip link to the main content region (excluding special cases)?</v>
+      <c r="C50" s="32" t="s">
+        <v>158</v>
       </c>
       <c r="D50" s="32" t="s">
         <v>73</v>
@@ -14379,14 +14285,13 @@
       <c r="BL50" s="48"/>
     </row>
     <row r="51" spans="1:64" s="49" customFormat="1" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A51" s="105"/>
+      <c r="A51" s="106"/>
       <c r="B51" s="46" t="str">
         <f>Criteria!B50</f>
         <v>12.8</v>
       </c>
-      <c r="C51" s="32" t="str">
-        <f>Criteria!C50</f>
-        <v>On each web page, is the navigation sequence consistent?</v>
+      <c r="C51" s="32" t="s">
+        <v>182</v>
       </c>
       <c r="D51" s="32" t="s">
         <v>73</v>
@@ -14455,14 +14360,13 @@
       <c r="BL51" s="48"/>
     </row>
     <row r="52" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A52" s="105"/>
+      <c r="A52" s="106"/>
       <c r="B52" s="46" t="str">
         <f>Criteria!B51</f>
         <v>12.9</v>
       </c>
-      <c r="C52" s="32" t="str">
-        <f>Criteria!C51</f>
-        <v>On each web page, navigation must not contain any keyboard traps. Is this rule respected?</v>
+      <c r="C52" s="32" t="s">
+        <v>159</v>
       </c>
       <c r="D52" s="32" t="s">
         <v>73</v>
@@ -14531,14 +14435,13 @@
       <c r="BL52" s="48"/>
     </row>
     <row r="53" spans="1:64" s="49" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A53" s="104"/>
+      <c r="A53" s="107"/>
       <c r="B53" s="84" t="str">
         <f>Criteria!B52</f>
         <v>12.11</v>
       </c>
-      <c r="C53" s="85" t="str">
-        <f>Criteria!C52</f>
-        <v>On each web page, is the additional content that appears when hovering over, focusing on or activating a user interface component accessible by keyboard if necessary?</v>
+      <c r="C53" s="85" t="s">
+        <v>160</v>
       </c>
       <c r="D53" s="32" t="s">
         <v>73</v>
@@ -14607,7 +14510,7 @@
       <c r="BL53" s="48"/>
     </row>
     <row r="54" spans="1:64" s="49" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A54" s="103" t="str">
+      <c r="A54" s="105" t="str">
         <f>Criteria!$A$53</f>
         <v>CONSULTATION</v>
       </c>
@@ -14615,9 +14518,8 @@
         <f>Criteria!B53</f>
         <v>13.1</v>
       </c>
-      <c r="C54" s="82" t="str">
-        <f>Criteria!C53</f>
-        <v>For each web page, does the user have control over each time limit for modifying the content (excluding special cases)?</v>
+      <c r="C54" s="82" t="s">
+        <v>161</v>
       </c>
       <c r="D54" s="32" t="s">
         <v>73</v>
@@ -14686,14 +14588,13 @@
       <c r="BL54" s="48"/>
     </row>
     <row r="55" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A55" s="105"/>
+      <c r="A55" s="106"/>
       <c r="B55" s="46" t="str">
         <f>Criteria!B54</f>
         <v>13.7</v>
       </c>
-      <c r="C55" s="32" t="str">
-        <f>Criteria!C54</f>
-        <v>On each web page, are sudden changes in brightness or blinking used correctly?</v>
+      <c r="C55" s="32" t="s">
+        <v>183</v>
       </c>
       <c r="D55" s="32" t="s">
         <v>73</v>
@@ -14762,14 +14663,13 @@
       <c r="BL55" s="48"/>
     </row>
     <row r="56" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A56" s="104"/>
+      <c r="A56" s="107"/>
       <c r="B56" s="84" t="str">
         <f>Criteria!B55</f>
         <v>13.8</v>
       </c>
-      <c r="C56" s="85" t="str">
-        <f>Criteria!C55</f>
-        <v>On each web page, is every moving or blinking content controllable by the user?</v>
+      <c r="C56" s="85" t="s">
+        <v>184</v>
       </c>
       <c r="D56" s="32" t="s">
         <v>73</v>
@@ -14839,6 +14739,12 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="A27:A34"/>
+    <mergeCell ref="A54:A56"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="A37:A41"/>
+    <mergeCell ref="A42:A48"/>
+    <mergeCell ref="A49:A53"/>
     <mergeCell ref="A14:A21"/>
     <mergeCell ref="A22:A23"/>
     <mergeCell ref="A24:A25"/>
@@ -14846,33 +14752,27 @@
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A4:A10"/>
     <mergeCell ref="A12:A13"/>
-    <mergeCell ref="A27:A34"/>
-    <mergeCell ref="A54:A56"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="A37:A41"/>
-    <mergeCell ref="A42:A48"/>
-    <mergeCell ref="A49:A53"/>
   </mergeCells>
+  <conditionalFormatting sqref="D4:D56">
+    <cfRule type="cellIs" dxfId="11" priority="5" operator="equal">
+      <formula>"C"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="10" priority="6" operator="equal">
+      <formula>"NC"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="9" priority="7" operator="equal">
+      <formula>"NA"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="8" priority="8" operator="equal">
+      <formula>"NT"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="E4:E56">
-    <cfRule type="cellIs" dxfId="11" priority="20" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="20" operator="equal">
       <formula>"D"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="21" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="21" operator="equal">
       <formula>"N"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D4:D56">
-    <cfRule type="cellIs" dxfId="9" priority="5" operator="equal">
-      <formula>"C"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="6" operator="equal">
-      <formula>"NC"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="7" operator="equal">
-      <formula>"NA"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="8" operator="equal">
-      <formula>"NT"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
@@ -15014,7 +14914,7 @@
       <c r="BL3" s="48"/>
     </row>
     <row r="4" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A4" s="103" t="str">
+      <c r="A4" s="105" t="str">
         <f>Criteria!$A$3</f>
         <v>IMAGES</v>
       </c>
@@ -15022,9 +14922,8 @@
         <f>Criteria!B3</f>
         <v>1.1</v>
       </c>
-      <c r="C4" s="82" t="str">
-        <f>Criteria!C3</f>
-        <v>Does each image conveying information have a text alternative?</v>
+      <c r="C4" s="32" t="s">
+        <v>125</v>
       </c>
       <c r="D4" s="82" t="s">
         <v>73</v>
@@ -15092,14 +14991,13 @@
       <c r="BL4" s="48"/>
     </row>
     <row r="5" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A5" s="105"/>
+      <c r="A5" s="106"/>
       <c r="B5" s="46" t="str">
         <f>Criteria!B4</f>
         <v>1.2</v>
       </c>
-      <c r="C5" s="32" t="str">
-        <f>Criteria!C4</f>
-        <v>Is every decorative image correctly ignored by assistive technologies?</v>
+      <c r="C5" s="32" t="s">
+        <v>126</v>
       </c>
       <c r="D5" s="82" t="s">
         <v>73</v>
@@ -15168,14 +15066,13 @@
       <c r="BL5" s="48"/>
     </row>
     <row r="6" spans="1:64" s="49" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A6" s="105"/>
+      <c r="A6" s="106"/>
       <c r="B6" s="46" t="str">
         <f>Criteria!B5</f>
         <v>1.3</v>
       </c>
-      <c r="C6" s="32" t="str">
-        <f>Criteria!C5</f>
-        <v>For each image conveying information with a text alternative, is this alternative relevant (excluding special cases)?</v>
+      <c r="C6" s="32" t="s">
+        <v>127</v>
       </c>
       <c r="D6" s="82" t="s">
         <v>73</v>
@@ -15244,14 +15141,13 @@
       <c r="BL6" s="48"/>
     </row>
     <row r="7" spans="1:64" s="49" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A7" s="105"/>
+      <c r="A7" s="106"/>
       <c r="B7" s="46" t="str">
         <f>Criteria!B6</f>
         <v>1.4</v>
       </c>
-      <c r="C7" s="32" t="str">
-        <f>Criteria!C6</f>
-        <v>For each image used as a CAPTCHA or test image, with a text alternative, does this alternative make it possible to identify the nature and function of the image?</v>
+      <c r="C7" s="32" t="s">
+        <v>128</v>
       </c>
       <c r="D7" s="82" t="s">
         <v>73</v>
@@ -15320,14 +15216,13 @@
       <c r="BL7" s="48"/>
     </row>
     <row r="8" spans="1:64" s="49" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A8" s="105"/>
+      <c r="A8" s="106"/>
       <c r="B8" s="46" t="str">
         <f>Criteria!B7</f>
         <v>1.5</v>
       </c>
-      <c r="C8" s="32" t="str">
-        <f>Criteria!C7</f>
-        <v>For each image used as a CAPTCHA, is there an alternative access solution to the content or to the CAPTCHA function?</v>
+      <c r="C8" s="32" t="s">
+        <v>129</v>
       </c>
       <c r="D8" s="82" t="s">
         <v>73</v>
@@ -15396,14 +15291,13 @@
       <c r="BL8" s="48"/>
     </row>
     <row r="9" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A9" s="105"/>
+      <c r="A9" s="106"/>
       <c r="B9" s="46" t="str">
         <f>Criteria!B8</f>
         <v>1.6</v>
       </c>
-      <c r="C9" s="32" t="str">
-        <f>Criteria!C8</f>
-        <v>Does each image conveying information have, if necessary, a detailed description?</v>
+      <c r="C9" s="32" t="s">
+        <v>130</v>
       </c>
       <c r="D9" s="82" t="s">
         <v>73</v>
@@ -15472,14 +15366,13 @@
       <c r="BL9" s="48"/>
     </row>
     <row r="10" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A10" s="104"/>
+      <c r="A10" s="107"/>
       <c r="B10" s="84" t="str">
         <f>Criteria!B9</f>
         <v>1.7</v>
       </c>
-      <c r="C10" s="85" t="str">
-        <f>Criteria!C9</f>
-        <v>For each image conveying information with a detailed description, is this description relevant?</v>
+      <c r="C10" s="75" t="s">
+        <v>131</v>
       </c>
       <c r="D10" s="82" t="s">
         <v>73</v>
@@ -15556,9 +15449,8 @@
         <f>Criteria!B10</f>
         <v>2.1</v>
       </c>
-      <c r="C11" s="80" t="str">
-        <f>Criteria!C10</f>
-        <v>Does each frame have a frame title?</v>
+      <c r="C11" s="80" t="s">
+        <v>132</v>
       </c>
       <c r="D11" s="82" t="s">
         <v>73</v>
@@ -15627,7 +15519,7 @@
       <c r="BL11" s="48"/>
     </row>
     <row r="12" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A12" s="103" t="str">
+      <c r="A12" s="105" t="str">
         <f>Criteria!$A$11</f>
         <v>COLOURS</v>
       </c>
@@ -15635,9 +15527,8 @@
         <f>Criteria!B11</f>
         <v>3.1</v>
       </c>
-      <c r="C12" s="82" t="str">
-        <f>Criteria!C11</f>
-        <v>On each web page, the information must not be provided by colour alone. Is this rule respected?</v>
+      <c r="C12" s="77" t="s">
+        <v>169</v>
       </c>
       <c r="D12" s="82" t="s">
         <v>73</v>
@@ -15706,14 +15597,13 @@
       <c r="BL12" s="48"/>
     </row>
     <row r="13" spans="1:64" s="49" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A13" s="104"/>
+      <c r="A13" s="107"/>
       <c r="B13" s="84" t="str">
         <f>Criteria!B12</f>
         <v>3.2</v>
       </c>
-      <c r="C13" s="85" t="str">
-        <f>Criteria!C12</f>
-        <v>On each web page, is the contrast between the colour of the text and the colour of its background sufficiently high (excluding special cases)?</v>
+      <c r="C13" s="75" t="s">
+        <v>133</v>
       </c>
       <c r="D13" s="82" t="s">
         <v>73</v>
@@ -15782,7 +15672,7 @@
       <c r="BL13" s="48"/>
     </row>
     <row r="14" spans="1:64" s="49" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A14" s="103" t="str">
+      <c r="A14" s="105" t="str">
         <f>Criteria!$A$13</f>
         <v>MULTIMEDIA</v>
       </c>
@@ -15790,9 +15680,8 @@
         <f>Criteria!B13</f>
         <v>4.1</v>
       </c>
-      <c r="C14" s="82" t="str">
-        <f>Criteria!C13</f>
-        <v>Does each pre-recorded time-based media have, if necessary, a transcript or an audio description (excluding special cases)?</v>
+      <c r="C14" s="82" t="s">
+        <v>134</v>
       </c>
       <c r="D14" s="82" t="s">
         <v>73</v>
@@ -15861,14 +15750,13 @@
       <c r="BL14" s="48"/>
     </row>
     <row r="15" spans="1:64" s="49" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A15" s="105"/>
+      <c r="A15" s="106"/>
       <c r="B15" s="46" t="str">
         <f>Criteria!B14</f>
         <v>4.2</v>
       </c>
-      <c r="C15" s="32" t="str">
-        <f>Criteria!C14</f>
-        <v>For each pre-recorded time-based media with a synchronised transcript or audio description, are these relevant (excluding special cases)?</v>
+      <c r="C15" s="32" t="s">
+        <v>135</v>
       </c>
       <c r="D15" s="82" t="s">
         <v>73</v>
@@ -15937,14 +15825,13 @@
       <c r="BL15" s="48"/>
     </row>
     <row r="16" spans="1:64" s="49" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A16" s="105"/>
+      <c r="A16" s="106"/>
       <c r="B16" s="46" t="str">
         <f>Criteria!B15</f>
         <v>4.3</v>
       </c>
-      <c r="C16" s="32" t="str">
-        <f>Criteria!C15</f>
-        <v>Does each pre-recorded synchronised time-based media have, if necessary, synchronised captions (excluding special cases)?</v>
+      <c r="C16" s="32" t="s">
+        <v>170</v>
       </c>
       <c r="D16" s="82" t="s">
         <v>73</v>
@@ -16013,14 +15900,13 @@
       <c r="BL16" s="48"/>
     </row>
     <row r="17" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A17" s="105"/>
+      <c r="A17" s="106"/>
       <c r="B17" s="46" t="str">
         <f>Criteria!B16</f>
         <v>4.4</v>
       </c>
-      <c r="C17" s="32" t="str">
-        <f>Criteria!C16</f>
-        <v>For each pre-recorded synchronised time-based media with synchronised subtitles, are these captions relevant?</v>
+      <c r="C17" s="32" t="s">
+        <v>171</v>
       </c>
       <c r="D17" s="82" t="s">
         <v>73</v>
@@ -16089,14 +15975,13 @@
       <c r="BL17" s="48"/>
     </row>
     <row r="18" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A18" s="105"/>
+      <c r="A18" s="106"/>
       <c r="B18" s="46" t="str">
         <f>Criteria!B17</f>
         <v>4.8</v>
       </c>
-      <c r="C18" s="32" t="str">
-        <f>Criteria!C17</f>
-        <v>Does each non-time-based media have, if necessary, an alternative (excluding special cases)?</v>
+      <c r="C18" s="32" t="s">
+        <v>136</v>
       </c>
       <c r="D18" s="82" t="s">
         <v>73</v>
@@ -16165,14 +16050,13 @@
       <c r="BL18" s="48"/>
     </row>
     <row r="19" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A19" s="105"/>
+      <c r="A19" s="106"/>
       <c r="B19" s="46" t="str">
         <f>Criteria!B18</f>
         <v>4.9</v>
       </c>
-      <c r="C19" s="32" t="str">
-        <f>Criteria!C18</f>
-        <v>For each non-time-based media having an alternative, is this alternative relevant?</v>
+      <c r="C19" s="32" t="s">
+        <v>137</v>
       </c>
       <c r="D19" s="82" t="s">
         <v>73</v>
@@ -16241,14 +16125,13 @@
       <c r="BL19" s="48"/>
     </row>
     <row r="20" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A20" s="105"/>
+      <c r="A20" s="106"/>
       <c r="B20" s="46" t="str">
         <f>Criteria!B19</f>
         <v>4.10</v>
       </c>
-      <c r="C20" s="32" t="str">
-        <f>Criteria!C19</f>
-        <v>Is each automatically triggered sound controllable by the user?</v>
+      <c r="C20" s="32" t="s">
+        <v>138</v>
       </c>
       <c r="D20" s="82" t="s">
         <v>73</v>
@@ -16317,14 +16200,13 @@
       <c r="BL20" s="48"/>
     </row>
     <row r="21" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A21" s="104"/>
+      <c r="A21" s="107"/>
       <c r="B21" s="84" t="str">
         <f>Criteria!B20</f>
         <v>4.11</v>
       </c>
-      <c r="C21" s="85" t="str">
-        <f>Criteria!C20</f>
-        <v>Is the viewing of each time-based media, if required, controllable by keyboard and any pointing device?</v>
+      <c r="C21" s="85" t="s">
+        <v>139</v>
       </c>
       <c r="D21" s="82" t="s">
         <v>73</v>
@@ -16393,16 +16275,15 @@
       <c r="BL21" s="48"/>
     </row>
     <row r="22" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A22" s="103" t="s">
+      <c r="A22" s="105" t="s">
         <v>26</v>
       </c>
       <c r="B22" s="81" t="str">
         <f>Criteria!B21</f>
         <v>5.6</v>
       </c>
-      <c r="C22" s="82" t="str">
-        <f>Criteria!C21</f>
-        <v>For each data table, are each column header and each row header correctly declared?</v>
+      <c r="C22" s="82" t="s">
+        <v>140</v>
       </c>
       <c r="D22" s="82" t="s">
         <v>73</v>
@@ -16471,14 +16352,13 @@
       <c r="BL22" s="48"/>
     </row>
     <row r="23" spans="1:64" s="49" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A23" s="104"/>
+      <c r="A23" s="107"/>
       <c r="B23" s="84" t="str">
         <f>Criteria!B22</f>
         <v>5.7</v>
       </c>
-      <c r="C23" s="85" t="str">
-        <f>Criteria!C22</f>
-        <v>For each data table, is the appropriate technique used to associate each cell with its headers (excluding special cases)?</v>
+      <c r="C23" s="85" t="s">
+        <v>141</v>
       </c>
       <c r="D23" s="82" t="s">
         <v>73</v>
@@ -16547,7 +16427,7 @@
       <c r="BL23" s="48"/>
     </row>
     <row r="24" spans="1:64" s="49" customFormat="1" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A24" s="103" t="str">
+      <c r="A24" s="105" t="str">
         <f>Criteria!$A$23</f>
         <v>LINKS</v>
       </c>
@@ -16555,9 +16435,8 @@
         <f>Criteria!B23</f>
         <v>6.1</v>
       </c>
-      <c r="C24" s="82" t="str">
-        <f>Criteria!C23</f>
-        <v>Is every link explicit (except in special cases)?</v>
+      <c r="C24" s="82" t="s">
+        <v>142</v>
       </c>
       <c r="D24" s="82" t="s">
         <v>73</v>
@@ -16626,14 +16505,13 @@
       <c r="BL24" s="48"/>
     </row>
     <row r="25" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A25" s="104"/>
+      <c r="A25" s="107"/>
       <c r="B25" s="84" t="str">
         <f>Criteria!B24</f>
         <v>6.2</v>
       </c>
-      <c r="C25" s="85" t="str">
-        <f>Criteria!C24</f>
-        <v>On each web page, does each link have an accessible name?</v>
+      <c r="C25" s="85" t="s">
+        <v>172</v>
       </c>
       <c r="D25" s="82" t="s">
         <v>73</v>
@@ -16709,9 +16587,8 @@
         <f>Criteria!B25</f>
         <v>7.3</v>
       </c>
-      <c r="C26" s="80" t="str">
-        <f>Criteria!C25</f>
-        <v>Is each script accessible and operable by keyboard and any pointing device (excluding special cases)?</v>
+      <c r="C26" s="80" t="s">
+        <v>173</v>
       </c>
       <c r="D26" s="82" t="s">
         <v>73</v>
@@ -16780,15 +16657,14 @@
       <c r="BL26" s="48"/>
     </row>
     <row r="27" spans="1:64" s="49" customFormat="1" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A27" s="106" t="s">
+      <c r="A27" s="103" t="s">
         <v>92</v>
       </c>
       <c r="B27" s="81">
         <v>8.1</v>
       </c>
-      <c r="C27" s="82" t="str">
-        <f>Criteria!C26</f>
-        <v>Has each web page a defined document type?</v>
+      <c r="C27" s="82" t="s">
+        <v>174</v>
       </c>
       <c r="D27" s="82" t="s">
         <v>73</v>
@@ -16857,14 +16733,13 @@
       <c r="BL27" s="48"/>
     </row>
     <row r="28" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A28" s="98"/>
+      <c r="A28" s="95"/>
       <c r="B28" s="46" t="str">
         <f>Criteria!B27</f>
         <v>8.2</v>
       </c>
-      <c r="C28" s="32" t="str">
-        <f>Criteria!C27</f>
-        <v>For each web page, is the generated source code valid for the specified document type?</v>
+      <c r="C28" s="32" t="s">
+        <v>143</v>
       </c>
       <c r="D28" s="82" t="s">
         <v>73</v>
@@ -16933,14 +16808,13 @@
       <c r="BL28" s="48"/>
     </row>
     <row r="29" spans="1:64" s="49" customFormat="1" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A29" s="98"/>
+      <c r="A29" s="95"/>
       <c r="B29" s="46" t="str">
         <f>Criteria!B28</f>
         <v>8.3</v>
       </c>
-      <c r="C29" s="32" t="str">
-        <f>Criteria!C28</f>
-        <v>On each web page, is the default language present?</v>
+      <c r="C29" s="32" t="s">
+        <v>144</v>
       </c>
       <c r="D29" s="82" t="s">
         <v>73</v>
@@ -17009,14 +16883,13 @@
       <c r="BL29" s="48"/>
     </row>
     <row r="30" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A30" s="98"/>
+      <c r="A30" s="95"/>
       <c r="B30" s="46" t="str">
         <f>Criteria!B29</f>
         <v>8.4</v>
       </c>
-      <c r="C30" s="32" t="str">
-        <f>Criteria!C29</f>
-        <v>For each web page with a default language, is the language code relevant?</v>
+      <c r="C30" s="32" t="s">
+        <v>145</v>
       </c>
       <c r="D30" s="82" t="s">
         <v>73</v>
@@ -17085,14 +16958,13 @@
       <c r="BL30" s="48"/>
     </row>
     <row r="31" spans="1:64" s="49" customFormat="1" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A31" s="98"/>
+      <c r="A31" s="95"/>
       <c r="B31" s="46" t="str">
         <f>Criteria!B30</f>
         <v>8.5</v>
       </c>
-      <c r="C31" s="32" t="str">
-        <f>Criteria!C30</f>
-        <v>Does every web page have a page title?</v>
+      <c r="C31" s="32" t="s">
+        <v>146</v>
       </c>
       <c r="D31" s="82" t="s">
         <v>73</v>
@@ -17161,14 +17033,13 @@
       <c r="BL31" s="48"/>
     </row>
     <row r="32" spans="1:64" s="49" customFormat="1" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A32" s="98"/>
+      <c r="A32" s="95"/>
       <c r="B32" s="46" t="str">
         <f>Criteria!B31</f>
         <v>8.6</v>
       </c>
-      <c r="C32" s="32" t="str">
-        <f>Criteria!C31</f>
-        <v>For each web page with a page title, is this title relevant?</v>
+      <c r="C32" s="32" t="s">
+        <v>147</v>
       </c>
       <c r="D32" s="82" t="s">
         <v>73</v>
@@ -17237,14 +17108,13 @@
       <c r="BL32" s="48"/>
     </row>
     <row r="33" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A33" s="98"/>
+      <c r="A33" s="95"/>
       <c r="B33" s="46" t="str">
         <f>Criteria!B32</f>
         <v>8.7</v>
       </c>
-      <c r="C33" s="32" t="str">
-        <f>Criteria!C32</f>
-        <v>On each web page, is each language change indicated in the source code (excluding special cases)?</v>
+      <c r="C33" s="32" t="s">
+        <v>148</v>
       </c>
       <c r="D33" s="82" t="s">
         <v>73</v>
@@ -17313,14 +17183,13 @@
       <c r="BL33" s="48"/>
     </row>
     <row r="34" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A34" s="107"/>
+      <c r="A34" s="104"/>
       <c r="B34" s="84" t="str">
         <f>Criteria!B33</f>
         <v>8.8</v>
       </c>
-      <c r="C34" s="85" t="str">
-        <f>Criteria!C33</f>
-        <v>On each web page, is the language code for each language change valid and relevant?</v>
+      <c r="C34" s="85" t="s">
+        <v>149</v>
       </c>
       <c r="D34" s="82" t="s">
         <v>73</v>
@@ -17389,7 +17258,7 @@
       <c r="BL34" s="48"/>
     </row>
     <row r="35" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A35" s="103" t="str">
+      <c r="A35" s="105" t="str">
         <f>Criteria!$A$34</f>
         <v>STRUCTURATION</v>
       </c>
@@ -17397,9 +17266,8 @@
         <f>Criteria!B34</f>
         <v>9.1</v>
       </c>
-      <c r="C35" s="82" t="str">
-        <f>Criteria!C34</f>
-        <v>On each web page, is the information structured by the appropriate use of headings?</v>
+      <c r="C35" s="82" t="s">
+        <v>175</v>
       </c>
       <c r="D35" s="82" t="s">
         <v>73</v>
@@ -17468,14 +17336,13 @@
       <c r="BL35" s="48"/>
     </row>
     <row r="36" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A36" s="104"/>
+      <c r="A36" s="107"/>
       <c r="B36" s="84" t="str">
         <f>Criteria!B35</f>
         <v>9.2</v>
       </c>
-      <c r="C36" s="85" t="str">
-        <f>Criteria!C35</f>
-        <v>On each web page, is the document structure consistent (excluding special cases)?</v>
+      <c r="C36" s="85" t="s">
+        <v>150</v>
       </c>
       <c r="D36" s="82" t="s">
         <v>73</v>
@@ -17544,16 +17411,15 @@
       <c r="BL36" s="48"/>
     </row>
     <row r="37" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A37" s="103" t="s">
+      <c r="A37" s="105" t="s">
         <v>93</v>
       </c>
       <c r="B37" s="81" t="str">
         <f>Criteria!B36</f>
         <v>10.7</v>
       </c>
-      <c r="C37" s="82" t="str">
-        <f>Criteria!C36</f>
-        <v>On each web page, for each element receiving the focus, is the focus visible?</v>
+      <c r="C37" s="82" t="s">
+        <v>151</v>
       </c>
       <c r="D37" s="82" t="s">
         <v>73</v>
@@ -17622,14 +17488,13 @@
       <c r="BL37" s="48"/>
     </row>
     <row r="38" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A38" s="105"/>
+      <c r="A38" s="106"/>
       <c r="B38" s="46" t="str">
         <f>Criteria!B37</f>
         <v>10.8</v>
       </c>
-      <c r="C38" s="32" t="str">
-        <f>Criteria!C37</f>
-        <v>For each web page, should hidden content be ignored by assistive technologies?</v>
+      <c r="C38" s="32" t="s">
+        <v>152</v>
       </c>
       <c r="D38" s="82" t="s">
         <v>73</v>
@@ -17698,14 +17563,13 @@
       <c r="BL38" s="48"/>
     </row>
     <row r="39" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A39" s="105"/>
+      <c r="A39" s="106"/>
       <c r="B39" s="46" t="str">
         <f>Criteria!B38</f>
         <v>10.9</v>
       </c>
-      <c r="C39" s="32" t="str">
-        <f>Criteria!C38</f>
-        <v>On each web page, information must not be conveyed solely by shape, size or location. Is this rule respected?</v>
+      <c r="C39" s="32" t="s">
+        <v>153</v>
       </c>
       <c r="D39" s="82" t="s">
         <v>73</v>
@@ -17774,14 +17638,13 @@
       <c r="BL39" s="48"/>
     </row>
     <row r="40" spans="1:64" s="49" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A40" s="105"/>
+      <c r="A40" s="106"/>
       <c r="B40" s="46" t="str">
         <f>Criteria!B39</f>
         <v>10.10</v>
       </c>
-      <c r="C40" s="32" t="str">
-        <f>Criteria!C39</f>
-        <v>On each web page, information must not be conveyed by shape, size or location only. Is this rule implemented appropriately?</v>
+      <c r="C40" s="32" t="s">
+        <v>154</v>
       </c>
       <c r="D40" s="82" t="s">
         <v>73</v>
@@ -17850,14 +17713,13 @@
       <c r="BL40" s="48"/>
     </row>
     <row r="41" spans="1:64" s="49" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A41" s="104"/>
+      <c r="A41" s="107"/>
       <c r="B41" s="84" t="str">
         <f>Criteria!B40</f>
         <v>10.14</v>
       </c>
-      <c r="C41" s="85" t="str">
-        <f>Criteria!C40</f>
-        <v>On each web page, can additional content that appears using CSS styles only be made visible using the keyboard and any pointing device?</v>
+      <c r="C41" s="85" t="s">
+        <v>155</v>
       </c>
       <c r="D41" s="82" t="s">
         <v>73</v>
@@ -17926,7 +17788,7 @@
       <c r="BL41" s="48"/>
     </row>
     <row r="42" spans="1:64" s="49" customFormat="1" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A42" s="103" t="str">
+      <c r="A42" s="105" t="str">
         <f>Criteria!$A$41</f>
         <v>FORMS</v>
       </c>
@@ -17934,9 +17796,8 @@
         <f>Criteria!B41</f>
         <v>11.1</v>
       </c>
-      <c r="C42" s="82" t="str">
-        <f>Criteria!C41</f>
-        <v>Does each form input field have a label?</v>
+      <c r="C42" s="82" t="s">
+        <v>156</v>
       </c>
       <c r="D42" s="82" t="s">
         <v>73</v>
@@ -18005,14 +17866,13 @@
       <c r="BL42" s="48"/>
     </row>
     <row r="43" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A43" s="105"/>
+      <c r="A43" s="106"/>
       <c r="B43" s="46" t="str">
         <f>Criteria!B42</f>
         <v>11.2</v>
       </c>
-      <c r="C43" s="32" t="str">
-        <f>Criteria!C42</f>
-        <v>Is each label associated with a form field relevant (excluding special cases)?</v>
+      <c r="C43" s="32" t="s">
+        <v>157</v>
       </c>
       <c r="D43" s="82" t="s">
         <v>73</v>
@@ -18081,14 +17941,13 @@
       <c r="BL43" s="48"/>
     </row>
     <row r="44" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A44" s="105"/>
+      <c r="A44" s="106"/>
       <c r="B44" s="46" t="str">
         <f>Criteria!B43</f>
         <v>11.5</v>
       </c>
-      <c r="C44" s="32" t="str">
-        <f>Criteria!C43</f>
-        <v>In each form, are the related form controls grouped together, if necessary?</v>
+      <c r="C44" s="32" t="s">
+        <v>176</v>
       </c>
       <c r="D44" s="82" t="s">
         <v>73</v>
@@ -18157,14 +18016,13 @@
       <c r="BL44" s="48"/>
     </row>
     <row r="45" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A45" s="105"/>
+      <c r="A45" s="106"/>
       <c r="B45" s="46" t="str">
         <f>Criteria!B44</f>
         <v>11.6</v>
       </c>
-      <c r="C45" s="32" t="str">
-        <f>Criteria!C44</f>
-        <v>In each form, does each group of related form controls have a legend?</v>
+      <c r="C45" s="32" t="s">
+        <v>177</v>
       </c>
       <c r="D45" s="82" t="s">
         <v>73</v>
@@ -18233,14 +18091,13 @@
       <c r="BL45" s="48"/>
     </row>
     <row r="46" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A46" s="105"/>
+      <c r="A46" s="106"/>
       <c r="B46" s="46" t="str">
         <f>Criteria!B45</f>
         <v>11.7</v>
       </c>
-      <c r="C46" s="32" t="str">
-        <f>Criteria!C45</f>
-        <v>In each form, is each legend associated with a group of related form controls relevant?</v>
+      <c r="C46" s="32" t="s">
+        <v>178</v>
       </c>
       <c r="D46" s="82" t="s">
         <v>73</v>
@@ -18309,14 +18166,13 @@
       <c r="BL46" s="48"/>
     </row>
     <row r="47" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A47" s="105"/>
+      <c r="A47" s="106"/>
       <c r="B47" s="46" t="str">
         <f>Criteria!B46</f>
         <v>11.9</v>
       </c>
-      <c r="C47" s="32" t="str">
-        <f>Criteria!C46</f>
-        <v>In each form, is the label of each button relevant (excluding special cases)?</v>
+      <c r="C47" s="32" t="s">
+        <v>179</v>
       </c>
       <c r="D47" s="82" t="s">
         <v>73</v>
@@ -18385,14 +18241,13 @@
       <c r="BL47" s="48"/>
     </row>
     <row r="48" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A48" s="104"/>
+      <c r="A48" s="107"/>
       <c r="B48" s="84" t="str">
         <f>Criteria!B47</f>
         <v>11.10</v>
       </c>
-      <c r="C48" s="85" t="str">
-        <f>Criteria!C47</f>
-        <v>In each form, is the error management used appropriately (excluding special cases)?</v>
+      <c r="C48" s="85" t="s">
+        <v>185</v>
       </c>
       <c r="D48" s="82" t="s">
         <v>73</v>
@@ -18461,16 +18316,15 @@
       <c r="BL48" s="48"/>
     </row>
     <row r="49" spans="1:64" s="49" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A49" s="103" t="s">
+      <c r="A49" s="105" t="s">
         <v>57</v>
       </c>
       <c r="B49" s="81" t="str">
         <f>Criteria!B48</f>
         <v>12.6</v>
       </c>
-      <c r="C49" s="82" t="str">
-        <f>Criteria!C48</f>
-        <v>Can content grouping regions present in several web pages header, main navigation, main content, footer and search engine) be reached or avoided?</v>
+      <c r="C49" s="82" t="s">
+        <v>186</v>
       </c>
       <c r="D49" s="82" t="s">
         <v>73</v>
@@ -18539,14 +18393,13 @@
       <c r="BL49" s="48"/>
     </row>
     <row r="50" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A50" s="105"/>
+      <c r="A50" s="106"/>
       <c r="B50" s="46" t="str">
         <f>Criteria!B49</f>
         <v>12.7</v>
       </c>
-      <c r="C50" s="32" t="str">
-        <f>Criteria!C49</f>
-        <v>On each web page, is there a bypass or skip link to the main content region (excluding special cases)?</v>
+      <c r="C50" s="32" t="s">
+        <v>158</v>
       </c>
       <c r="D50" s="82" t="s">
         <v>73</v>
@@ -18615,14 +18468,13 @@
       <c r="BL50" s="48"/>
     </row>
     <row r="51" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A51" s="105"/>
+      <c r="A51" s="106"/>
       <c r="B51" s="46" t="str">
         <f>Criteria!B50</f>
         <v>12.8</v>
       </c>
-      <c r="C51" s="32" t="str">
-        <f>Criteria!C50</f>
-        <v>On each web page, is the navigation sequence consistent?</v>
+      <c r="C51" s="32" t="s">
+        <v>182</v>
       </c>
       <c r="D51" s="82" t="s">
         <v>73</v>
@@ -18691,14 +18543,13 @@
       <c r="BL51" s="48"/>
     </row>
     <row r="52" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A52" s="105"/>
+      <c r="A52" s="106"/>
       <c r="B52" s="46" t="str">
         <f>Criteria!B51</f>
         <v>12.9</v>
       </c>
-      <c r="C52" s="32" t="str">
-        <f>Criteria!C51</f>
-        <v>On each web page, navigation must not contain any keyboard traps. Is this rule respected?</v>
+      <c r="C52" s="32" t="s">
+        <v>159</v>
       </c>
       <c r="D52" s="82" t="s">
         <v>73</v>
@@ -18767,14 +18618,13 @@
       <c r="BL52" s="48"/>
     </row>
     <row r="53" spans="1:64" s="49" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A53" s="104"/>
+      <c r="A53" s="107"/>
       <c r="B53" s="84" t="str">
         <f>Criteria!B52</f>
         <v>12.11</v>
       </c>
-      <c r="C53" s="85" t="str">
-        <f>Criteria!C52</f>
-        <v>On each web page, is the additional content that appears when hovering over, focusing on or activating a user interface component accessible by keyboard if necessary?</v>
+      <c r="C53" s="85" t="s">
+        <v>160</v>
       </c>
       <c r="D53" s="82" t="s">
         <v>73</v>
@@ -18843,7 +18693,7 @@
       <c r="BL53" s="48"/>
     </row>
     <row r="54" spans="1:64" s="49" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A54" s="103" t="str">
+      <c r="A54" s="105" t="str">
         <f>Criteria!$A$53</f>
         <v>CONSULTATION</v>
       </c>
@@ -18851,9 +18701,8 @@
         <f>Criteria!B53</f>
         <v>13.1</v>
       </c>
-      <c r="C54" s="82" t="str">
-        <f>Criteria!C53</f>
-        <v>For each web page, does the user have control over each time limit for modifying the content (excluding special cases)?</v>
+      <c r="C54" s="82" t="s">
+        <v>161</v>
       </c>
       <c r="D54" s="82" t="s">
         <v>73</v>
@@ -18922,14 +18771,13 @@
       <c r="BL54" s="48"/>
     </row>
     <row r="55" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A55" s="105"/>
+      <c r="A55" s="106"/>
       <c r="B55" s="46" t="str">
         <f>Criteria!B54</f>
         <v>13.7</v>
       </c>
-      <c r="C55" s="32" t="str">
-        <f>Criteria!C54</f>
-        <v>On each web page, are sudden changes in brightness or blinking used correctly?</v>
+      <c r="C55" s="32" t="s">
+        <v>183</v>
       </c>
       <c r="D55" s="82" t="s">
         <v>73</v>
@@ -18998,14 +18846,13 @@
       <c r="BL55" s="48"/>
     </row>
     <row r="56" spans="1:64" s="49" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A56" s="104"/>
+      <c r="A56" s="107"/>
       <c r="B56" s="84" t="str">
         <f>Criteria!B55</f>
         <v>13.8</v>
       </c>
-      <c r="C56" s="85" t="str">
-        <f>Criteria!C55</f>
-        <v>On each web page, is every moving or blinking content controllable by the user?</v>
+      <c r="C56" s="85" t="s">
+        <v>184</v>
       </c>
       <c r="D56" s="82" t="s">
         <v>73</v>
@@ -19075,6 +18922,12 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="A27:A34"/>
+    <mergeCell ref="A54:A56"/>
+    <mergeCell ref="A35:A36"/>
+    <mergeCell ref="A37:A41"/>
+    <mergeCell ref="A42:A48"/>
+    <mergeCell ref="A49:A53"/>
     <mergeCell ref="A14:A21"/>
     <mergeCell ref="A22:A23"/>
     <mergeCell ref="A24:A25"/>
@@ -19082,12 +18935,6 @@
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A4:A10"/>
     <mergeCell ref="A12:A13"/>
-    <mergeCell ref="A27:A34"/>
-    <mergeCell ref="A54:A56"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="A37:A41"/>
-    <mergeCell ref="A42:A48"/>
-    <mergeCell ref="A49:A53"/>
   </mergeCells>
   <conditionalFormatting sqref="D4:D56">
     <cfRule type="cellIs" dxfId="5" priority="8" operator="equal">

</xml_diff>